<commit_message>
Revise CLOs to eight outcomes aligned with the BCS_AD program
- Merge ER design and relational mapping into one design CLO (CLO2); renumber
  the rest so the eight CLOs fill the template's CLO rows
- Update CLO references in the schedule, grading structure, and draft materials
- Expand the council brief with CLO derivation, Bloom distribution, alignment
  with the 9-semester program, CLO-assessment matrix, preliminary PLO areas,
  and anticipated questions about the CLOs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157NQpBHkydaVuWPpDtVnkB
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -2488,7 +2488,7 @@
       </c>
       <c r="C2" s="104" t="inlineStr">
         <is>
-          <t>Explain the fundamental concepts of database systems (data models, schemas, the three-schema architecture, data independence) and trace how they arose from the research literature.</t>
+          <t>Explain the fundamental concepts of database systems (data models, schemas and instances, the three-schema architecture, data independence, DBMS components) and relate them to the research contributions that introduced them.</t>
         </is>
       </c>
       <c r="D2" s="103" t="n"/>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="C3" s="104" t="inlineStr">
         <is>
-          <t>Design Entity-Relationship models from requirements, compare design alternatives, and identify constraints that the ER model cannot express.</t>
+          <t>Design a database from requirements: build an Entity-Relationship model, justify design alternatives, and map it to a relational schema whose keys and integrity constraints are specified precisely, including as logical statements.</t>
         </is>
       </c>
       <c r="D3" s="103" t="n"/>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C4" s="104" t="inlineStr">
         <is>
-          <t>Map ER models to relational schemas and state keys, foreign keys and other integrity constraints precisely, including as logical statements.</t>
+          <t>Formulate queries in relational algebra and relational calculus, prove simple equivalences between expressions, and explain the limits of their expressive power.</t>
         </is>
       </c>
       <c r="D4" s="103" t="n"/>
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C5" s="104" t="inlineStr">
         <is>
-          <t>Express queries in relational algebra and relational calculus, prove simple equivalences, and reason about the expressive power of query languages.</t>
+          <t>Use SQL to define, populate, modify and query relational databases (joins, aggregation, subqueries, views, access from Python) and explain query results through SQL semantics (bag semantics, three-valued logic).</t>
         </is>
       </c>
       <c r="D5" s="103" t="n"/>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="C6" s="104" t="inlineStr">
         <is>
-          <t>Write SQL to define, modify and query databases (joins, aggregation, subqueries, views, access from Python) and explain its semantics (bags, three-valued logic) by translation to algebra.</t>
+          <t>Analyze and improve relational schemas with functional dependency theory: compute closures, candidate keys and minimal covers, prove basic properties, decompose to 3NF/BCNF with lossless-join and dependency-preservation guarantees, and implement these algorithms in Python.</t>
         </is>
       </c>
       <c r="D6" s="103" t="n"/>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="C7" s="104" t="inlineStr">
         <is>
-          <t>Apply functional dependency theory: compute closures, keys and minimal covers, prove properties, normalize to 3NF/BCNF, verify lossless-join and dependency preservation, and implement these algorithms in Python.</t>
+          <t>Evaluate physical design and query execution choices (storage organization, indexes, join algorithms, execution plans) using I/O cost models and controlled experiments.</t>
         </is>
       </c>
       <c r="D7" s="103" t="n"/>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="C8" s="104" t="inlineStr">
         <is>
-          <t>Analyze storage, indexing, query processing and optimization with I/O cost models, and evaluate index and plan choices experimentally.</t>
+          <t>Analyze concurrent executions for conflict serializability and recoverability, and justify concurrency-control and recovery mechanisms (two-phase locking, isolation levels, write-ahead logging).</t>
         </is>
       </c>
       <c r="D8" s="103" t="n"/>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="C9" s="104" t="inlineStr">
         <is>
-          <t>Analyze schedules for conflict serializability and recoverability, explain locking, isolation levels and logging-based recovery, and justify the correctness of two-phase locking.</t>
+          <t>Conduct a small, reproducible research study on a database topic: review primary literature, formulate a research question or hypothesis, design and carry out an experiment or implementation, and report the results in an academic paper and presentation.</t>
         </is>
       </c>
       <c r="D9" s="103" t="n"/>
@@ -2741,20 +2741,10 @@
       <c r="T9" s="103" t="n"/>
       <c r="U9" s="103" t="n"/>
     </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="129" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="130" t="inlineStr">
-        <is>
-          <t>CLO9</t>
-        </is>
-      </c>
-      <c r="C10" s="104" t="inlineStr">
-        <is>
-          <t>Conduct a small research study in databases: read primary literature, formulate a question or hypothesis, design a reproducible experiment or implementation, and report the results in an academic format.</t>
-        </is>
-      </c>
+    <row r="10">
+      <c r="A10" s="103" t="n"/>
+      <c r="B10" s="103" t="n"/>
+      <c r="C10" s="103" t="n"/>
       <c r="D10" s="103" t="n"/>
       <c r="E10" s="103" t="n"/>
       <c r="F10" s="103" t="n"/>
@@ -3100,31 +3090,17 @@
       <c r="U21" s="113" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="131" t="inlineStr">
-        <is>
-          <t>CLO9</t>
-        </is>
-      </c>
-      <c r="B22" s="106" t="n"/>
-      <c r="C22" s="107" t="n"/>
-      <c r="D22" s="106" t="n"/>
+      <c r="A22" s="103" t="n"/>
+      <c r="B22" s="103" t="n"/>
+      <c r="C22" s="103" t="n"/>
+      <c r="D22" s="103" t="n"/>
       <c r="E22" s="103" t="n"/>
       <c r="F22" s="103" t="n"/>
       <c r="G22" s="103" t="n"/>
       <c r="H22" s="103" t="n"/>
       <c r="I22" s="103" t="n"/>
       <c r="J22" s="103" t="n"/>
-      <c r="K22" s="106" t="n"/>
-      <c r="L22" s="113" t="n"/>
-      <c r="M22" s="113" t="n"/>
-      <c r="N22" s="113" t="n"/>
-      <c r="O22" s="113" t="n"/>
-      <c r="P22" s="113" t="n"/>
-      <c r="Q22" s="113" t="n"/>
-      <c r="R22" s="113" t="n"/>
-      <c r="S22" s="113" t="n"/>
-      <c r="T22" s="113" t="n"/>
-      <c r="U22" s="113" t="n"/>
+      <c r="K22" s="103" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="103" t="n"/>
@@ -4846,7 +4822,7 @@
       </c>
       <c r="D10" s="32" t="inlineStr">
         <is>
-          <t>CLO3</t>
+          <t>CLO2</t>
         </is>
       </c>
       <c r="E10" s="32" t="inlineStr">
@@ -4897,7 +4873,7 @@
       </c>
       <c r="D11" s="32" t="inlineStr">
         <is>
-          <t>CLO3</t>
+          <t>CLO2</t>
         </is>
       </c>
       <c r="E11" s="32" t="inlineStr">
@@ -4951,7 +4927,7 @@
       </c>
       <c r="D12" s="32" t="inlineStr">
         <is>
-          <t>CLO3</t>
+          <t>CLO2</t>
         </is>
       </c>
       <c r="E12" s="32" t="inlineStr">
@@ -5002,7 +4978,7 @@
       </c>
       <c r="D13" s="32" t="inlineStr">
         <is>
-          <t>CLO3</t>
+          <t>CLO2</t>
         </is>
       </c>
       <c r="E13" s="32" t="inlineStr">
@@ -5057,7 +5033,7 @@
       </c>
       <c r="D14" s="32" t="inlineStr">
         <is>
-          <t>CLO2, CLO3</t>
+          <t>CLO2</t>
         </is>
       </c>
       <c r="E14" s="32" t="inlineStr">
@@ -5108,7 +5084,7 @@
       </c>
       <c r="D15" s="32" t="inlineStr">
         <is>
-          <t>CLO4</t>
+          <t>CLO3</t>
         </is>
       </c>
       <c r="E15" s="32" t="inlineStr">
@@ -5158,7 +5134,7 @@
       </c>
       <c r="D16" s="32" t="inlineStr">
         <is>
-          <t>CLO4</t>
+          <t>CLO3</t>
         </is>
       </c>
       <c r="E16" s="32" t="inlineStr">
@@ -5219,7 +5195,7 @@
       </c>
       <c r="D17" s="32" t="inlineStr">
         <is>
-          <t>CLO4</t>
+          <t>CLO3</t>
         </is>
       </c>
       <c r="E17" s="32" t="inlineStr">
@@ -5271,7 +5247,7 @@
       </c>
       <c r="D18" s="32" t="inlineStr">
         <is>
-          <t>CLO4</t>
+          <t>CLO3</t>
         </is>
       </c>
       <c r="E18" s="32" t="inlineStr">
@@ -5321,7 +5297,7 @@
       </c>
       <c r="D19" s="32" t="inlineStr">
         <is>
-          <t>CLO4</t>
+          <t>CLO3</t>
         </is>
       </c>
       <c r="E19" s="32" t="inlineStr">
@@ -5370,7 +5346,7 @@
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
-          <t>CLO1, CLO2, CLO3, CLO4</t>
+          <t>CLO1, CLO2, CLO3</t>
         </is>
       </c>
       <c r="E20" s="32" t="inlineStr">
@@ -5419,7 +5395,7 @@
       </c>
       <c r="D21" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E21" s="32" t="inlineStr">
@@ -5470,7 +5446,7 @@
       </c>
       <c r="D22" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E22" s="32" t="inlineStr">
@@ -5521,7 +5497,7 @@
       </c>
       <c r="D23" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E23" s="32" t="inlineStr">
@@ -5571,7 +5547,7 @@
       </c>
       <c r="D24" s="32" t="inlineStr">
         <is>
-          <t>CLO3, CLO5</t>
+          <t>CLO2, CLO4</t>
         </is>
       </c>
       <c r="E24" s="32" t="inlineStr">
@@ -5619,7 +5595,7 @@
       </c>
       <c r="D25" s="32" t="inlineStr">
         <is>
-          <t>CLO3, CLO5</t>
+          <t>CLO2, CLO4</t>
         </is>
       </c>
       <c r="E25" s="32" t="inlineStr">
@@ -5667,7 +5643,7 @@
       </c>
       <c r="D26" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E26" s="32" t="inlineStr">
@@ -5718,7 +5694,7 @@
       </c>
       <c r="D27" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E27" s="32" t="inlineStr">
@@ -5768,7 +5744,7 @@
       </c>
       <c r="D28" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E28" s="32" t="inlineStr">
@@ -5818,7 +5794,7 @@
       </c>
       <c r="D29" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E29" s="32" t="inlineStr">
@@ -5865,7 +5841,7 @@
       </c>
       <c r="D30" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E30" s="32" t="inlineStr">
@@ -5915,7 +5891,7 @@
       </c>
       <c r="D31" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E31" s="32" t="inlineStr">
@@ -5966,7 +5942,7 @@
       </c>
       <c r="D32" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E32" s="32" t="inlineStr">
@@ -6016,7 +5992,7 @@
       </c>
       <c r="D33" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E33" s="32" t="inlineStr">
@@ -6063,7 +6039,7 @@
       </c>
       <c r="D34" s="32" t="inlineStr">
         <is>
-          <t>CLO4, CLO5</t>
+          <t>CLO3, CLO4</t>
         </is>
       </c>
       <c r="E34" s="32" t="inlineStr">
@@ -6110,7 +6086,7 @@
       </c>
       <c r="D35" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E35" s="32" t="inlineStr">
@@ -6161,7 +6137,7 @@
       </c>
       <c r="D36" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E36" s="32" t="inlineStr">
@@ -6211,7 +6187,7 @@
       </c>
       <c r="D37" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E37" s="32" t="inlineStr">
@@ -6261,7 +6237,7 @@
       </c>
       <c r="D38" s="32" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E38" s="32" t="inlineStr">
@@ -6308,7 +6284,7 @@
       </c>
       <c r="D39" s="32" t="inlineStr">
         <is>
-          <t>CLO2, CLO3, CLO4, CLO9</t>
+          <t>CLO2, CLO3, CLO8</t>
         </is>
       </c>
       <c r="E39" s="32" t="inlineStr">
@@ -6356,7 +6332,7 @@
       </c>
       <c r="D40" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E40" s="32" t="inlineStr">
@@ -6406,7 +6382,7 @@
       </c>
       <c r="D41" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E41" s="32" t="inlineStr">
@@ -6457,7 +6433,7 @@
       </c>
       <c r="D42" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E42" s="32" t="inlineStr">
@@ -6507,7 +6483,7 @@
       </c>
       <c r="D43" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E43" s="32" t="inlineStr">
@@ -6557,7 +6533,7 @@
       </c>
       <c r="D44" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E44" s="32" t="inlineStr">
@@ -6609,7 +6585,7 @@
       </c>
       <c r="D45" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E45" s="32" t="inlineStr">
@@ -6659,7 +6635,7 @@
       </c>
       <c r="D46" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E46" s="32" t="inlineStr">
@@ -6708,7 +6684,7 @@
       </c>
       <c r="D47" s="32" t="inlineStr">
         <is>
-          <t>CLO5, CLO6</t>
+          <t>CLO4, CLO5</t>
         </is>
       </c>
       <c r="E47" s="32" t="inlineStr">
@@ -6756,7 +6732,7 @@
       </c>
       <c r="D48" s="32" t="inlineStr">
         <is>
-          <t>CLO7</t>
+          <t>CLO6</t>
         </is>
       </c>
       <c r="E48" s="32" t="inlineStr">
@@ -6806,7 +6782,7 @@
       </c>
       <c r="D49" s="32" t="inlineStr">
         <is>
-          <t>CLO7</t>
+          <t>CLO6</t>
         </is>
       </c>
       <c r="E49" s="32" t="inlineStr">
@@ -6857,7 +6833,7 @@
       </c>
       <c r="D50" s="32" t="inlineStr">
         <is>
-          <t>CLO7</t>
+          <t>CLO6</t>
         </is>
       </c>
       <c r="E50" s="32" t="inlineStr">
@@ -6909,7 +6885,7 @@
       </c>
       <c r="D51" s="32" t="inlineStr">
         <is>
-          <t>CLO7</t>
+          <t>CLO6</t>
         </is>
       </c>
       <c r="E51" s="32" t="inlineStr">
@@ -6960,7 +6936,7 @@
       </c>
       <c r="D52" s="32" t="inlineStr">
         <is>
-          <t>CLO7, CLO9</t>
+          <t>CLO6, CLO8</t>
         </is>
       </c>
       <c r="E52" s="32" t="inlineStr">
@@ -7011,7 +6987,7 @@
       </c>
       <c r="D53" s="32" t="inlineStr">
         <is>
-          <t>CLO8</t>
+          <t>CLO7</t>
         </is>
       </c>
       <c r="E53" s="32" t="inlineStr">
@@ -7062,7 +7038,7 @@
       </c>
       <c r="D54" s="32" t="inlineStr">
         <is>
-          <t>CLO8</t>
+          <t>CLO7</t>
         </is>
       </c>
       <c r="E54" s="32" t="inlineStr">
@@ -7114,7 +7090,7 @@
       </c>
       <c r="D55" s="32" t="inlineStr">
         <is>
-          <t>CLO8</t>
+          <t>CLO7</t>
         </is>
       </c>
       <c r="E55" s="32" t="inlineStr">
@@ -7166,7 +7142,7 @@
       </c>
       <c r="D56" s="32" t="inlineStr">
         <is>
-          <t>CLO8</t>
+          <t>CLO7</t>
         </is>
       </c>
       <c r="E56" s="32" t="inlineStr">
@@ -7216,7 +7192,7 @@
       </c>
       <c r="D57" s="32" t="inlineStr">
         <is>
-          <t>CLO8</t>
+          <t>CLO7</t>
         </is>
       </c>
       <c r="E57" s="32" t="inlineStr">
@@ -7264,7 +7240,7 @@
       </c>
       <c r="D58" s="32" t="inlineStr">
         <is>
-          <t>CLO9</t>
+          <t>CLO8</t>
         </is>
       </c>
       <c r="E58" s="32" t="inlineStr">
@@ -7311,7 +7287,7 @@
       </c>
       <c r="D59" s="32" t="inlineStr">
         <is>
-          <t>CLO7, CLO8, CLO9</t>
+          <t>CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="E59" s="32" t="inlineStr">
@@ -7358,7 +7334,7 @@
       </c>
       <c r="D60" s="32" t="inlineStr">
         <is>
-          <t>CLO7, CLO8, CLO9</t>
+          <t>CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="E60" s="32" t="inlineStr">
@@ -7406,7 +7382,7 @@
       </c>
       <c r="D61" s="32" t="inlineStr">
         <is>
-          <t>CLO1–CLO9</t>
+          <t>CLO1–CLO8</t>
         </is>
       </c>
       <c r="E61" s="32" t="inlineStr">
@@ -7644,7 +7620,7 @@
       </c>
       <c r="H3" s="72" t="inlineStr">
         <is>
-          <t>CLO1, CLO2, CLO3, CLO4</t>
+          <t>CLO1, CLO2, CLO3</t>
         </is>
       </c>
       <c r="I3" s="25" t="inlineStr">
@@ -7711,7 +7687,7 @@
       </c>
       <c r="H4" s="72" t="inlineStr">
         <is>
-          <t>CLO5, CLO6</t>
+          <t>CLO4, CLO5</t>
         </is>
       </c>
       <c r="I4" s="25" t="inlineStr">
@@ -7778,7 +7754,7 @@
       </c>
       <c r="H5" s="72" t="inlineStr">
         <is>
-          <t>CLO2, CLO3, CLO4, CLO9</t>
+          <t>CLO2, CLO3, CLO8</t>
         </is>
       </c>
       <c r="I5" s="25" t="inlineStr">
@@ -7841,7 +7817,7 @@
       </c>
       <c r="H6" s="72" t="inlineStr">
         <is>
-          <t>CLO6, CLO7, CLO8, CLO9</t>
+          <t>CLO5, CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="I6" s="25" t="inlineStr">
@@ -7904,7 +7880,7 @@
       </c>
       <c r="H7" s="72" t="inlineStr">
         <is>
-          <t>CLO5</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="I7" s="25" t="inlineStr">
@@ -7967,7 +7943,7 @@
       </c>
       <c r="H8" s="72" t="inlineStr">
         <is>
-          <t>CLO1, CLO2, CLO3, CLO4, CLO5, CLO6, CLO7, CLO8</t>
+          <t>CLO1, CLO2, CLO3, CLO4, CLO5, CLO6, CLO7</t>
         </is>
       </c>
       <c r="I8" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Map CLOs to the 13 BCS_AD PLOs
- Fill the CLO-PLO matrix in the syllabus workbook with the template's tick style
- Add the mapping to syllabus.md
- Council brief: PLO summaries, mapping matrix, rationale and evidence for each
  link, PLOs not claimed and why, and related anticipated questions
- Keep the PLO source file under syllabus/template/

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157NQpBHkydaVuWPpDtVnkB
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -583,7 +583,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -949,6 +949,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2767,7 +2773,7 @@
     <row r="11">
       <c r="A11" s="120" t="inlineStr">
         <is>
-          <t>Mapping of CLOs to PLOs of Curriculum BCS_AD (K22A) – to be completed when the program PLO list is confirmed</t>
+          <t>Mapping of CLOs to PLOs of Curriculum BCS_AD (K22A, 13 PLOs)</t>
         </is>
       </c>
     </row>
@@ -2849,26 +2855,10 @@
           <t>PLO13</t>
         </is>
       </c>
-      <c r="O13" s="105" t="inlineStr">
-        <is>
-          <t>PLO14</t>
-        </is>
-      </c>
-      <c r="P13" s="105" t="inlineStr">
-        <is>
-          <t>PLO15</t>
-        </is>
-      </c>
-      <c r="Q13" s="105" t="inlineStr">
-        <is>
-          <t>PLO16</t>
-        </is>
-      </c>
-      <c r="R13" s="105" t="inlineStr">
-        <is>
-          <t>PLO17</t>
-        </is>
-      </c>
+      <c r="O13" s="105" t="n"/>
+      <c r="P13" s="105" t="n"/>
+      <c r="Q13" s="105" t="n"/>
+      <c r="R13" s="105" t="n"/>
       <c r="S13" s="105" t="n"/>
       <c r="T13" s="105" t="n"/>
       <c r="U13" s="105" t="n"/>
@@ -2880,7 +2870,11 @@
         </is>
       </c>
       <c r="B14" s="106" t="n"/>
-      <c r="C14" s="107" t="n"/>
+      <c r="C14" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D14" s="106" t="n"/>
       <c r="E14" s="103" t="n"/>
       <c r="F14" s="103" t="n"/>
@@ -2907,10 +2901,18 @@
         </is>
       </c>
       <c r="B15" s="106" t="n"/>
-      <c r="C15" s="107" t="n"/>
+      <c r="C15" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D15" s="106" t="n"/>
       <c r="E15" s="103" t="n"/>
-      <c r="F15" s="103" t="n"/>
+      <c r="F15" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="G15" s="103" t="n"/>
       <c r="H15" s="103" t="n"/>
       <c r="I15" s="103" t="n"/>
@@ -2934,10 +2936,18 @@
         </is>
       </c>
       <c r="B16" s="106" t="n"/>
-      <c r="C16" s="107" t="n"/>
+      <c r="C16" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D16" s="106" t="n"/>
       <c r="E16" s="103" t="n"/>
-      <c r="F16" s="103" t="n"/>
+      <c r="F16" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="G16" s="103" t="n"/>
       <c r="H16" s="103" t="n"/>
       <c r="I16" s="103" t="n"/>
@@ -2961,13 +2971,21 @@
         </is>
       </c>
       <c r="B17" s="106" t="n"/>
-      <c r="C17" s="107" t="n"/>
+      <c r="C17" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D17" s="106" t="n"/>
       <c r="E17" s="103" t="n"/>
       <c r="F17" s="103" t="n"/>
       <c r="G17" s="103" t="n"/>
       <c r="H17" s="103" t="n"/>
-      <c r="I17" s="103" t="n"/>
+      <c r="I17" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="J17" s="103" t="n"/>
       <c r="K17" s="106" t="n"/>
       <c r="L17" s="113" t="n"/>
@@ -2988,13 +3006,25 @@
         </is>
       </c>
       <c r="B18" s="106" t="n"/>
-      <c r="C18" s="107" t="n"/>
+      <c r="C18" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D18" s="106" t="n"/>
       <c r="E18" s="103" t="n"/>
-      <c r="F18" s="103" t="n"/>
+      <c r="F18" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="G18" s="103" t="n"/>
       <c r="H18" s="103" t="n"/>
-      <c r="I18" s="103" t="n"/>
+      <c r="I18" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="J18" s="103" t="n"/>
       <c r="K18" s="106" t="n"/>
       <c r="L18" s="113" t="n"/>
@@ -3015,14 +3045,26 @@
         </is>
       </c>
       <c r="B19" s="106" t="n"/>
-      <c r="C19" s="107" t="n"/>
+      <c r="C19" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D19" s="106" t="n"/>
       <c r="E19" s="103" t="n"/>
-      <c r="F19" s="103" t="n"/>
+      <c r="F19" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="G19" s="103" t="n"/>
       <c r="H19" s="103" t="n"/>
       <c r="I19" s="103" t="n"/>
-      <c r="J19" s="103" t="n"/>
+      <c r="J19" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="K19" s="106" t="n"/>
       <c r="L19" s="113" t="n"/>
       <c r="M19" s="113" t="n"/>
@@ -3042,7 +3084,11 @@
         </is>
       </c>
       <c r="B20" s="106" t="n"/>
-      <c r="C20" s="107" t="n"/>
+      <c r="C20" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="D20" s="106" t="n"/>
       <c r="E20" s="103" t="n"/>
       <c r="F20" s="103" t="n"/>
@@ -3069,16 +3115,32 @@
         </is>
       </c>
       <c r="B21" s="106" t="n"/>
-      <c r="C21" s="107" t="n"/>
+      <c r="C21" s="132" t="n"/>
       <c r="D21" s="106" t="n"/>
       <c r="E21" s="103" t="n"/>
-      <c r="F21" s="103" t="n"/>
+      <c r="F21" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="G21" s="103" t="n"/>
-      <c r="H21" s="103" t="n"/>
+      <c r="H21" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="I21" s="103" t="n"/>
       <c r="J21" s="103" t="n"/>
-      <c r="K21" s="106" t="n"/>
-      <c r="L21" s="113" t="n"/>
+      <c r="K21" s="132" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
+      <c r="L21" s="133" t="inlineStr">
+        <is>
+          <t>ü</t>
+        </is>
+      </c>
       <c r="M21" s="113" t="n"/>
       <c r="N21" s="113" t="n"/>
       <c r="O21" s="113" t="n"/>
@@ -3222,594 +3284,594 @@
       </c>
     </row>
     <row r="2" ht="13.8" customHeight="1">
-      <c r="A2" s="132" t="n">
+      <c r="A2" s="134" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="133" t="n">
+      <c r="B2" s="135" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="134" t="inlineStr">
+      <c r="C2" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D2" s="135" t="inlineStr">
+      <c r="D2" s="137" t="inlineStr">
         <is>
           <t>Codd separated the logical view of data from its physical storage. What would be lost if applications had to know how and where each record is stored?</t>
         </is>
       </c>
     </row>
     <row r="3" ht="13.8" customHeight="1">
-      <c r="A3" s="132" t="n">
+      <c r="A3" s="134" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="133" t="n">
+      <c r="B3" s="135" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="134" t="inlineStr">
+      <c r="C3" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D3" s="135" t="inlineStr">
+      <c r="D3" s="137" t="inlineStr">
         <is>
           <t>Why do new data models (XML, document, graph, vector) keep appearing, and why do many of them end up adding SQL-like features?</t>
         </is>
       </c>
     </row>
     <row r="4" ht="13.8" customHeight="1">
-      <c r="A4" s="132" t="n">
+      <c r="A4" s="134" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="133" t="n">
+      <c r="B4" s="135" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="134" t="inlineStr">
+      <c r="C4" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D4" s="135" t="inlineStr">
+      <c r="D4" s="137" t="inlineStr">
         <is>
           <t>When is a database system NOT the right tool? Give a concrete example and justify it.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="13.8" customHeight="1">
-      <c r="A5" s="132" t="n">
+      <c r="A5" s="134" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="133" t="n">
+      <c r="B5" s="135" t="n">
         <v>7</v>
       </c>
-      <c r="C5" s="134" t="inlineStr">
+      <c r="C5" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D5" s="135" t="inlineStr">
+      <c r="D5" s="137" t="inlineStr">
         <is>
           <t>Why is Grade an attribute of the enrollment relationship and not of STUDENT or SECTION? What goes wrong if it is placed on either entity?</t>
         </is>
       </c>
     </row>
     <row r="6" ht="13.8" customHeight="1">
-      <c r="A6" s="132" t="n">
+      <c r="A6" s="134" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="133" t="n">
+      <c r="B6" s="135" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="134" t="inlineStr">
+      <c r="C6" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D6" s="135" t="inlineStr">
+      <c r="D6" s="137" t="inlineStr">
         <is>
           <t>Is a ternary relationship always equivalent to three binary relationships? Construct a counterexample.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="13.8" customHeight="1">
-      <c r="A7" s="132" t="n">
+      <c r="A7" s="134" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="133" t="n">
+      <c r="B7" s="135" t="n">
         <v>7</v>
       </c>
-      <c r="C7" s="134" t="inlineStr">
+      <c r="C7" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D7" s="135" t="inlineStr">
+      <c r="D7" s="137" t="inlineStr">
         <is>
           <t>Give a business rule of UniversityDB that cannot be drawn in an ER diagram. How should a designer record and enforce it?</t>
         </is>
       </c>
     </row>
     <row r="8" ht="13.8" customHeight="1">
-      <c r="A8" s="132" t="n">
+      <c r="A8" s="134" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="133" t="n">
+      <c r="B8" s="135" t="n">
         <v>12</v>
       </c>
-      <c r="C8" s="134" t="inlineStr">
+      <c r="C8" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D8" s="135" t="inlineStr">
+      <c r="D8" s="137" t="inlineStr">
         <is>
           <t>What would break if relations were allowed to contain duplicate tuples? Consider keys, projection and the meaning of a fact.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="13.8" customHeight="1">
-      <c r="A9" s="132" t="n">
+      <c r="A9" s="134" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="133" t="n">
+      <c r="B9" s="135" t="n">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="inlineStr">
+      <c r="C9" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D9" s="135" t="inlineStr">
+      <c r="D9" s="137" t="inlineStr">
         <is>
           <t>Why is NULL allowed in a foreign key but not in a primary key? Argue from what each constraint means.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="13.8" customHeight="1">
-      <c r="A10" s="132" t="n">
+      <c r="A10" s="134" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="133" t="n">
+      <c r="B10" s="135" t="n">
         <v>12</v>
       </c>
-      <c r="C10" s="134" t="inlineStr">
+      <c r="C10" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D10" s="135" t="inlineStr">
+      <c r="D10" s="137" t="inlineStr">
         <is>
           <t>A 1:1 relationship can be mapped with a foreign key on either side, or by merging the two relations. How would you decide, and what evidence would you use?</t>
         </is>
       </c>
     </row>
     <row r="11" ht="13.8" customHeight="1">
-      <c r="A11" s="132" t="n">
+      <c r="A11" s="134" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="133" t="n">
+      <c r="B11" s="135" t="n">
         <v>17</v>
       </c>
-      <c r="C11" s="134" t="inlineStr">
+      <c r="C11" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D11" s="135" t="inlineStr">
+      <c r="D11" s="137" t="inlineStr">
         <is>
           <t>Why does projection remove duplicates in relational algebra while SELECT in SQL does not? What are the costs and benefits of each choice?</t>
         </is>
       </c>
     </row>
     <row r="12" ht="13.8" customHeight="1">
-      <c r="A12" s="132" t="n">
+      <c r="A12" s="134" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="133" t="n">
+      <c r="B12" s="135" t="n">
         <v>17</v>
       </c>
-      <c r="C12" s="134" t="inlineStr">
+      <c r="C12" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D12" s="135" t="inlineStr">
+      <c r="D12" s="137" t="inlineStr">
         <is>
           <t>Division expresses 'for all' queries. Why is there no basic 'for all' operator, and how does calculus express the same idea?</t>
         </is>
       </c>
     </row>
     <row r="13" ht="13.8" customHeight="1">
-      <c r="A13" s="132" t="n">
+      <c r="A13" s="134" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="133" t="n">
+      <c r="B13" s="135" t="n">
         <v>17</v>
       </c>
-      <c r="C13" s="134" t="inlineStr">
+      <c r="C13" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D13" s="135" t="inlineStr">
+      <c r="D13" s="137" t="inlineStr">
         <is>
           <t>Relational algebra cannot compute the transitive closure of a relation. Why does a fixed-size expression limit what a language can express?</t>
         </is>
       </c>
     </row>
     <row r="14" ht="13.8" customHeight="1">
-      <c r="A14" s="132" t="n">
+      <c r="A14" s="134" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="133" t="n">
+      <c r="B14" s="135" t="n">
         <v>22</v>
       </c>
-      <c r="C14" s="134" t="inlineStr">
+      <c r="C14" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D14" s="135" t="inlineStr">
+      <c r="D14" s="137" t="inlineStr">
         <is>
           <t>Why should integrity rules be declared in the database rather than checked in application code? When is the opposite true?</t>
         </is>
       </c>
     </row>
     <row r="15" ht="13.8" customHeight="1">
-      <c r="A15" s="132" t="n">
+      <c r="A15" s="134" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="133" t="n">
+      <c r="B15" s="135" t="n">
         <v>22</v>
       </c>
-      <c r="C15" s="134" t="inlineStr">
+      <c r="C15" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D15" s="135" t="inlineStr">
+      <c r="D15" s="137" t="inlineStr">
         <is>
           <t>Why do almost no DBMSs implement CREATE ASSERTION, although it is in the SQL standard?</t>
         </is>
       </c>
     </row>
     <row r="16" ht="13.8" customHeight="1">
-      <c r="A16" s="132" t="n">
+      <c r="A16" s="134" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="133" t="n">
+      <c r="B16" s="135" t="n">
         <v>22</v>
       </c>
-      <c r="C16" s="134" t="inlineStr">
+      <c r="C16" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D16" s="135" t="inlineStr">
+      <c r="D16" s="137" t="inlineStr">
         <is>
           <t>ON DELETE CASCADE is convenient. What risks does it create, and how could a cascade chain surprise a user?</t>
         </is>
       </c>
     </row>
     <row r="17" ht="13.8" customHeight="1">
-      <c r="A17" s="132" t="n">
+      <c r="A17" s="134" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="133" t="n">
+      <c r="B17" s="135" t="n">
         <v>26</v>
       </c>
-      <c r="C17" s="134" t="inlineStr">
+      <c r="C17" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D17" s="135" t="inlineStr">
+      <c r="D17" s="137" t="inlineStr">
         <is>
           <t>Under three-valued logic, 'p OR NOT p' is not always true. Which everyday query mistakes follow from this?</t>
         </is>
       </c>
     </row>
     <row r="18" ht="13.8" customHeight="1">
-      <c r="A18" s="132" t="n">
+      <c r="A18" s="134" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="133" t="n">
+      <c r="B18" s="135" t="n">
         <v>26</v>
       </c>
-      <c r="C18" s="134" t="inlineStr">
+      <c r="C18" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D18" s="135" t="inlineStr">
+      <c r="D18" s="137" t="inlineStr">
         <is>
           <t>Why does 'x NOT IN (subquery)' return no rows when the subquery contains NULL, while NOT EXISTS behaves differently?</t>
         </is>
       </c>
     </row>
     <row r="19" ht="13.8" customHeight="1">
-      <c r="A19" s="132" t="n">
+      <c r="A19" s="134" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="133" t="n">
+      <c r="B19" s="135" t="n">
         <v>26</v>
       </c>
-      <c r="C19" s="134" t="inlineStr">
+      <c r="C19" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D19" s="135" t="inlineStr">
+      <c r="D19" s="137" t="inlineStr">
         <is>
           <t>Which algebraic laws that hold for sets fail for bags? Why did SQL choose bag semantics anyway?</t>
         </is>
       </c>
     </row>
     <row r="20" ht="13.8" customHeight="1">
-      <c r="A20" s="132" t="n">
+      <c r="A20" s="134" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="133" t="n">
+      <c r="B20" s="135" t="n">
         <v>31</v>
       </c>
-      <c r="C20" s="134" t="inlineStr">
+      <c r="C20" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D20" s="135" t="inlineStr">
+      <c r="D20" s="137" t="inlineStr">
         <is>
           <t>A correlated subquery is evaluated 'once per outer row' in the textbook model. How could a DBMS evaluate it more efficiently?</t>
         </is>
       </c>
     </row>
     <row r="21" ht="13.8" customHeight="1">
-      <c r="A21" s="132" t="n">
+      <c r="A21" s="134" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="133" t="n">
+      <c r="B21" s="135" t="n">
         <v>31</v>
       </c>
-      <c r="C21" s="134" t="inlineStr">
+      <c r="C21" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D21" s="135" t="inlineStr">
+      <c r="D21" s="137" t="inlineStr">
         <is>
           <t>The same query can often be written with a join, a subquery or a set operation. Should the choice affect performance? Why or why not?</t>
         </is>
       </c>
     </row>
     <row r="22" ht="13.8" customHeight="1">
-      <c r="A22" s="132" t="n">
+      <c r="A22" s="134" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="133" t="n">
+      <c r="B22" s="135" t="n">
         <v>31</v>
       </c>
-      <c r="C22" s="134" t="inlineStr">
+      <c r="C22" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D22" s="135" t="inlineStr">
+      <c r="D22" s="137" t="inlineStr">
         <is>
           <t>Why did it take until 2017 to give SQL a complete formal semantics?</t>
         </is>
       </c>
     </row>
     <row r="23" ht="13.8" customHeight="1">
-      <c r="A23" s="132" t="n">
+      <c r="A23" s="134" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="133" t="n">
+      <c r="B23" s="135" t="n">
         <v>35</v>
       </c>
-      <c r="C23" s="134" t="inlineStr">
+      <c r="C23" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D23" s="135" t="inlineStr">
+      <c r="D23" s="137" t="inlineStr">
         <is>
           <t>Deleting a row through a join view can be translated in more than one way. Which translation should the DBMS choose, and why?</t>
         </is>
       </c>
     </row>
     <row r="24" ht="13.8" customHeight="1">
-      <c r="A24" s="132" t="n">
+      <c r="A24" s="134" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="133" t="n">
+      <c r="B24" s="135" t="n">
         <v>35</v>
       </c>
-      <c r="C24" s="134" t="inlineStr">
+      <c r="C24" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D24" s="135" t="inlineStr">
+      <c r="D24" s="137" t="inlineStr">
         <is>
           <t>A view costs nothing extra at run time. How is that possible?</t>
         </is>
       </c>
     </row>
     <row r="25" ht="13.8" customHeight="1">
-      <c r="A25" s="132" t="n">
+      <c r="A25" s="134" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="133" t="n">
+      <c r="B25" s="135" t="n">
         <v>35</v>
       </c>
-      <c r="C25" s="134" t="inlineStr">
+      <c r="C25" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D25" s="135" t="inlineStr">
+      <c r="D25" s="137" t="inlineStr">
         <is>
           <t>Why do parameterized queries prevent SQL injection, while escaping user input is considered fragile?</t>
         </is>
       </c>
     </row>
     <row r="26" ht="13.8" customHeight="1">
-      <c r="A26" s="132" t="n">
+      <c r="A26" s="134" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="133" t="n">
+      <c r="B26" s="135" t="n">
         <v>44</v>
       </c>
-      <c r="C26" s="134" t="inlineStr">
+      <c r="C26" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D26" s="135" t="inlineStr">
+      <c r="D26" s="137" t="inlineStr">
         <is>
           <t>Every normal form can be seen as removing one kind of redundancy. What single idea unifies them?</t>
         </is>
       </c>
     </row>
     <row r="27" ht="13.8" customHeight="1">
-      <c r="A27" s="132" t="n">
+      <c r="A27" s="134" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="133" t="n">
+      <c r="B27" s="135" t="n">
         <v>44</v>
       </c>
-      <c r="C27" s="134" t="inlineStr">
+      <c r="C27" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D27" s="135" t="inlineStr">
+      <c r="D27" s="137" t="inlineStr">
         <is>
           <t>BCNF decomposition may lose a dependency. When would you accept 3NF instead, and what do you gain?</t>
         </is>
       </c>
     </row>
     <row r="28" ht="13.8" customHeight="1">
-      <c r="A28" s="132" t="n">
+      <c r="A28" s="134" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="133" t="n">
+      <c r="B28" s="135" t="n">
         <v>44</v>
       </c>
-      <c r="C28" s="134" t="inlineStr">
+      <c r="C28" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D28" s="135" t="inlineStr">
+      <c r="D28" s="137" t="inlineStr">
         <is>
           <t>Testing whether an attribute is prime is NP-complete. What does this mean for automatic schema design tools?</t>
         </is>
       </c>
     </row>
     <row r="29" ht="13.8" customHeight="1">
-      <c r="A29" s="132" t="n">
+      <c r="A29" s="134" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="133" t="n">
+      <c r="B29" s="135" t="n">
         <v>50</v>
       </c>
-      <c r="C29" s="134" t="inlineStr">
+      <c r="C29" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D29" s="135" t="inlineStr">
+      <c r="D29" s="137" t="inlineStr">
         <is>
           <t>Why is a B-tree node the size of a disk page instead of holding a single key as in a binary search tree?</t>
         </is>
       </c>
     </row>
     <row r="30" ht="13.8" customHeight="1">
-      <c r="A30" s="132" t="n">
+      <c r="A30" s="134" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="133" t="n">
+      <c r="B30" s="135" t="n">
         <v>50</v>
       </c>
-      <c r="C30" s="134" t="inlineStr">
+      <c r="C30" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D30" s="135" t="inlineStr">
+      <c r="D30" s="137" t="inlineStr">
         <is>
           <t>The optimizer relies on estimates. What happens when the estimates are wrong, and where do the errors come from?</t>
         </is>
       </c>
     </row>
     <row r="31" ht="13.8" customHeight="1">
-      <c r="A31" s="132" t="n">
+      <c r="A31" s="134" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="133" t="n">
+      <c r="B31" s="135" t="n">
         <v>50</v>
       </c>
-      <c r="C31" s="134" t="inlineStr">
+      <c r="C31" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D31" s="135" t="inlineStr">
+      <c r="D31" s="137" t="inlineStr">
         <is>
           <t>Could a machine-learning model replace an index? What would you need to measure to decide?</t>
         </is>
       </c>
     </row>
     <row r="32" ht="13.8" customHeight="1">
-      <c r="A32" s="132" t="n">
+      <c r="A32" s="134" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="133" t="n">
+      <c r="B32" s="135" t="n">
         <v>55</v>
       </c>
-      <c r="C32" s="134" t="inlineStr">
+      <c r="C32" s="136" t="inlineStr">
         <is>
           <t>CQ1</t>
         </is>
       </c>
-      <c r="D32" s="135" t="inlineStr">
+      <c r="D32" s="137" t="inlineStr">
         <is>
           <t>Why is serializability the accepted correctness criterion for concurrent transactions? What weaker criteria do real systems use, and why?</t>
         </is>
       </c>
     </row>
     <row r="33" ht="13.8" customHeight="1">
-      <c r="A33" s="132" t="n">
+      <c r="A33" s="134" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="133" t="n">
+      <c r="B33" s="135" t="n">
         <v>55</v>
       </c>
-      <c r="C33" s="134" t="inlineStr">
+      <c r="C33" s="136" t="inlineStr">
         <is>
           <t>CQ2</t>
         </is>
       </c>
-      <c r="D33" s="135" t="inlineStr">
+      <c r="D33" s="137" t="inlineStr">
         <is>
           <t>Why does two-phase locking guarantee serializability? Explain the idea of the lock point.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="13.8" customHeight="1">
-      <c r="A34" s="132" t="n">
+      <c r="A34" s="134" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="133" t="n">
+      <c r="B34" s="135" t="n">
         <v>55</v>
       </c>
-      <c r="C34" s="134" t="inlineStr">
+      <c r="C34" s="136" t="inlineStr">
         <is>
           <t>CQ3</t>
         </is>
       </c>
-      <c r="D34" s="135" t="inlineStr">
+      <c r="D34" s="137" t="inlineStr">
         <is>
           <t>Snapshot isolation prevents dirty reads, non-repeatable reads and phantoms. Why is it still not serializable?</t>
         </is>
@@ -7977,7 +8039,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="136" t="inlineStr">
+      <c r="B9" s="138" t="inlineStr">
         <is>
           <t>Total</t>
         </is>

</xml_diff>

<commit_message>
Use the short objectives list as the syllabus Description
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157NQpBHkydaVuWPpDtVnkB
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -1583,7 +1583,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="190" customFormat="1" customHeight="1" s="10">
+    <row r="12" ht="125" customFormat="1" customHeight="1" s="10">
       <c r="A12" s="78" t="n">
         <v>11</v>
       </c>
@@ -1595,7 +1595,14 @@
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>This course gives a rigorous, research-oriented introduction to database systems for talented first-year Computer Science students. Students model data with the Entity-Relationship model and map it to the relational model, which is studied as a mathematical structure. They express queries in relational algebra, relational calculus and SQL, and reason about the semantics and expressive power of these languages. Functional dependency theory is developed with proofs and algorithms and applied to normalization. The course then opens the DBMS: storage and indexing under an I/O cost model, query processing and optimization, and the theory of transactions, concurrency control and recovery. Every chapter includes a 'Research Corner' built around a seminal paper, and students implement core algorithms in Python and carry out reproducible experiments. At the end of the course, students can design normalized schemas, query databases proficiently in SQL, explain the internal mechanisms of storage and transaction control, and conduct and report a small research study in the database field.</t>
+          <t>This course aims to help students:
+- understand the basic concepts of database systems and the relational model;
+- design databases with the Entity-Relationship model and convert them into relational schemas;
+- write queries in relational algebra, relational calculus and SQL;
+- use functional dependencies to evaluate and normalize a database design;
+- explain how a DBMS stores data, uses indexes and processes queries;
+- explain how transactions, concurrency control and recovery keep data correct;
+- read research papers and carry out small experiments on database topics.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace the Research Corner with graded constructivist-question answers
- Each student answers one constructivist question per chapter (150-200 words),
  graded 4% inside a 10% 'Labs and constructivist questions' component
- Remove Research Corner lines and papers from the syllabus; keep DSC, DMS, T-SQL
- Lighten per-session student tasks; mark the 10 CQ discussion sessions
- Update the council brief, design notes and project context

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157NQpBHkydaVuWPpDtVnkB
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -1602,7 +1602,7 @@
 - use functional dependencies to evaluate and normalize a database design;
 - explain how a DBMS stores data, uses indexes and processes queries;
 - explain how transactions, concurrency control and recovery keep data correct;
-- read research papers and carry out small experiments on database topics.</t>
+- answer research-style questions and carry out small experiments on database topics.</t>
         </is>
       </c>
     </row>
@@ -1619,8 +1619,9 @@
       <c r="C13" s="18" t="inlineStr">
         <is>
           <t>- Students must attend at least 80% of contact slots in order to be accepted to the final examination.
-- Read the assigned textbook sections and the Research Corner paper BEFORE each theory session, and prepare answers to the constructivist questions.
-- Complete all 9 research labs, including the 'Investigate' part and the Python implementation tasks, and submit them on time.
+- Read the assigned textbook sections BEFORE each theory session.
+- For each chapter, choose ONE of its three constructivist questions and submit a short written answer (150–200 words) on the LMS within one week of the discussion session. The answers are graded as part of the research score (4% in total).
+- Complete all 9 labs, including the 'Investigate' part and the Python implementation tasks, and submit them on time.
 - Complete Assignment 1 (individual technical report) and Assignment 2 (group mini research project: short paper, reproducible code and presentation).
 - Complete the guided self-study readings listed in the schedule (abstract topics such as relational calculus, statistics estimation and recovery algorithms); they are assessed in the progress tests and the final exam.
 - Keep all code, scripts and measurements in a version-controlled repository so that results are reproducible.
@@ -1663,7 +1664,7 @@
       <c r="C15" s="21" t="inlineStr">
         <is>
           <t>1) On-going Assessment
-- 9 Research labs:                        10%
+- 9 labs + 10 CQ answers:              10%
 - 2 Progress tests:                        20%
 - Assignment 1 (technical report):   10%
 - Assignment 2 (research project):  20%
@@ -1674,7 +1675,7 @@
 1) Every on-going assessment component &gt; 0
 2) Practical Exam &gt; 0
 3) Final Exam Score &gt;= 4 &amp; Final Result &gt;= 5
-Rationale: the course serves talented students on an academic track, so 40% of the grade rewards research work (labs, report, research project), 60% rewards individual mastery of theory and skills (progress tests, practical exam, final exam), and the final exam includes at least 30% analysis-level items.</t>
+Rationale: the course serves talented students on an academic track, so 40% of the grade rewards research work (labs, constructivist questions, report, research project), 60% rewards individual mastery of theory and skills (progress tests, practical exam, final exam), and the final exam includes at least 30% analysis-level items.</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="13.2"/>
   <cols>
     <col width="3.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2013,7 +2014,7 @@
       </c>
       <c r="B4" s="127" t="inlineStr">
         <is>
-          <t>What Goes Around Comes Around… And Around…</t>
+          <t>Transact-SQL reference</t>
         </is>
       </c>
       <c r="C4" s="128" t="inlineStr">
@@ -2029,445 +2030,66 @@
       </c>
       <c r="F4" s="127" t="inlineStr">
         <is>
-          <t>Research Corner, Chapter 1. ACM SIGMOD Record 53(2)</t>
+          <t>https://learn.microsoft.com/sql/t-sql/</t>
         </is>
       </c>
       <c r="G4" s="127" t="inlineStr">
         <is>
-          <t>Michael Stonebraker, Andrew Pavlo</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="H4" s="127" t="inlineStr">
         <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I4" s="127" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="I4" s="127" t="inlineStr"/>
       <c r="J4" s="127" t="inlineStr"/>
     </row>
-    <row r="5">
-      <c r="A5" s="127" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="127" t="inlineStr">
-        <is>
-          <t>A Relational Model of Data for Large Shared Data Banks</t>
-        </is>
-      </c>
-      <c r="C5" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D5" s="128" t="inlineStr"/>
-      <c r="E5" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F5" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 2. Communications of the ACM 13(6):377–387</t>
-        </is>
-      </c>
-      <c r="G5" s="127" t="inlineStr">
-        <is>
-          <t>E. F. Codd</t>
-        </is>
-      </c>
-      <c r="H5" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I5" s="127" t="inlineStr">
-        <is>
-          <t>1970</t>
-        </is>
-      </c>
-      <c r="J5" s="127" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="127" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="127" t="inlineStr">
-        <is>
-          <t>SEQUEL: A Structured English Query Language</t>
-        </is>
-      </c>
-      <c r="C6" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D6" s="128" t="inlineStr"/>
-      <c r="E6" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F6" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 3. Proc. ACM SIGFIDET Workshop</t>
-        </is>
-      </c>
-      <c r="G6" s="127" t="inlineStr">
-        <is>
-          <t>Donald D. Chamberlin, Raymond F. Boyce</t>
-        </is>
-      </c>
-      <c r="H6" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I6" s="127" t="inlineStr">
-        <is>
-          <t>1974</t>
-        </is>
-      </c>
-      <c r="J6" s="127" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="127" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="127" t="inlineStr">
-        <is>
-          <t>The Entity-Relationship Model—Toward a Unified View of Data</t>
-        </is>
-      </c>
-      <c r="C7" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D7" s="128" t="inlineStr"/>
-      <c r="E7" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F7" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 5. ACM TODS 1(1):9–36</t>
-        </is>
-      </c>
-      <c r="G7" s="127" t="inlineStr">
-        <is>
-          <t>Peter P. Chen</t>
-        </is>
-      </c>
-      <c r="H7" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I7" s="127" t="inlineStr">
-        <is>
-          <t>1976</t>
-        </is>
-      </c>
-      <c r="J7" s="127" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="127" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="127" t="inlineStr">
-        <is>
-          <t>A Simple Guide to Five Normal Forms in Relational Database Theory</t>
-        </is>
-      </c>
-      <c r="C8" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D8" s="128" t="inlineStr"/>
-      <c r="E8" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F8" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 6. Communications of the ACM 26(2):120–125</t>
-        </is>
-      </c>
-      <c r="G8" s="127" t="inlineStr">
-        <is>
-          <t>William Kent</t>
-        </is>
-      </c>
-      <c r="H8" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I8" s="127" t="inlineStr">
-        <is>
-          <t>1983</t>
-        </is>
-      </c>
-      <c r="J8" s="127" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" s="127" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="127" t="inlineStr">
-        <is>
-          <t>Organization and Maintenance of Large Ordered Indexes</t>
-        </is>
-      </c>
-      <c r="C9" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D9" s="128" t="inlineStr"/>
-      <c r="E9" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F9" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 7. Acta Informatica 1:173–189</t>
-        </is>
-      </c>
-      <c r="G9" s="127" t="inlineStr">
-        <is>
-          <t>Rudolf Bayer, Edward McCreight</t>
-        </is>
-      </c>
-      <c r="H9" s="127" t="inlineStr">
-        <is>
-          <t>Springer</t>
-        </is>
-      </c>
-      <c r="I9" s="127" t="inlineStr">
-        <is>
-          <t>1972</t>
-        </is>
-      </c>
-      <c r="J9" s="127" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="127" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="127" t="inlineStr">
-        <is>
-          <t>The Case for Learned Index Structures</t>
-        </is>
-      </c>
-      <c r="C10" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D10" s="128" t="inlineStr"/>
-      <c r="E10" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F10" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 7. Proc. ACM SIGMOD</t>
-        </is>
-      </c>
-      <c r="G10" s="127" t="inlineStr">
-        <is>
-          <t>T. Kraska, A. Beutel, E. H. Chi, J. Dean, N. Polyzotis</t>
-        </is>
-      </c>
-      <c r="H10" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I10" s="127" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="J10" s="127" t="inlineStr"/>
-    </row>
+      <c r="B9" s="119" t="inlineStr">
+        <is>
+          <t>Ghi rõ ISBN với sách hardcopy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11" ht="26.4" customHeight="1">
-      <c r="A11" s="127" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="127" t="inlineStr">
-        <is>
-          <t>Access Path Selection in a Relational Database Management System</t>
-        </is>
-      </c>
-      <c r="C11" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D11" s="128" t="inlineStr"/>
-      <c r="E11" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F11" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 8. Proc. ACM SIGMOD</t>
-        </is>
-      </c>
-      <c r="G11" s="127" t="inlineStr">
-        <is>
-          <t>P. G. Selinger et al.</t>
-        </is>
-      </c>
-      <c r="H11" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I11" s="127" t="inlineStr">
-        <is>
-          <t>1979</t>
-        </is>
-      </c>
-      <c r="J11" s="127" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="127" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="127" t="inlineStr">
-        <is>
-          <t>A Critique of ANSI SQL Isolation Levels</t>
-        </is>
-      </c>
-      <c r="C12" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D12" s="128" t="inlineStr"/>
-      <c r="E12" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F12" s="127" t="inlineStr">
-        <is>
-          <t>Research Corner, Chapter 9. Proc. ACM SIGMOD</t>
-        </is>
-      </c>
-      <c r="G12" s="127" t="inlineStr">
-        <is>
-          <t>H. Berenson et al.</t>
-        </is>
-      </c>
-      <c r="H12" s="127" t="inlineStr">
-        <is>
-          <t>ACM</t>
-        </is>
-      </c>
-      <c r="I12" s="127" t="inlineStr">
-        <is>
-          <t>1995</t>
-        </is>
-      </c>
-      <c r="J12" s="127" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="127" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="127" t="inlineStr">
-        <is>
-          <t>Transact-SQL reference</t>
-        </is>
-      </c>
-      <c r="C13" s="128" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D13" s="128" t="inlineStr"/>
-      <c r="E13" s="127" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
-      <c r="F13" s="127" t="inlineStr">
-        <is>
-          <t>https://learn.microsoft.com/sql/t-sql/</t>
-        </is>
-      </c>
-      <c r="G13" s="127" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="H13" s="127" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="I13" s="127" t="inlineStr"/>
-      <c r="J13" s="127" t="inlineStr"/>
-    </row>
-    <row r="14" ht="26.4" customHeight="1">
-      <c r="B14" s="117" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="116" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="119" t="inlineStr">
-        <is>
-          <t>Ghi rõ ISBN với sách hardcopy</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="114" t="inlineStr">
+      <c r="B11" s="114" t="inlineStr">
         <is>
           <t>Purpose: textbook or reference
 Type: hardcopy or online</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="116" t="inlineStr">
+      <c r="C11" s="118" t="n"/>
+    </row>
+    <row r="12">
+      <c r="C12" s="113" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="116" t="inlineStr">
         <is>
           <t>Đối với các môn "m" hoặc "c"</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="117" t="inlineStr">
+    <row r="14" ht="26.4" customHeight="1">
+      <c r="B14" s="117" t="inlineStr">
         <is>
           <t>MaterialDescription: Tên MOOC, 
                                   Eg. MOOC 1: Architecting Solutions on AWS</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="116" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="116" t="inlineStr">
         <is>
           <t>Author: Tên Trường/Côngty/Tổ chức biên soạn MOOC</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="116" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="116" t="inlineStr">
         <is>
           <t>Publisher: Coursera</t>
         </is>
@@ -4490,12 +4112,12 @@
       </c>
       <c r="H2" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 1, §1.1–1.3, pp. 1–12 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 1, §1.1–1.3, pp. 1–12 before class</t>
         </is>
       </c>
       <c r="I2" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 1; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 1</t>
         </is>
       </c>
       <c r="J2" s="115" t="inlineStr">
@@ -4551,13 +4173,13 @@
       </c>
       <c r="H3" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 1, §1.4–1.7, pp. 13–23 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 1, §1.4–1.7, pp. 13–23 before class
 Self-study: DSC §1.8–1.9 (users and administrators; history of database systems), pp. 24–28</t>
         </is>
       </c>
       <c r="I3" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 1; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 1</t>
         </is>
       </c>
       <c r="J3" s="115" t="n"/>
@@ -4569,7 +4191,7 @@
       </c>
       <c r="B4" s="32" t="inlineStr">
         <is>
-          <t>Research Corner: history of data models (Stonebraker &amp; Pavlo, 2024)
+          <t>Discussion of the Chapter 1 constructivist questions
 Lab 1: install SQL Server; load the sample university database</t>
         </is>
       </c>
@@ -4592,7 +4214,6 @@
       <c r="F4" s="33" t="inlineStr">
         <is>
           <t>- Slides: Chapter 1
-- Paper: Stonebraker &amp; Pavlo (2024)
 - Lab 1 handout
 - Textbook: DSC Appendix A, pp. 1287–1298</t>
         </is>
@@ -4605,12 +4226,13 @@
       </c>
       <c r="H4" s="31" t="inlineStr">
         <is>
-          <t>Read the paper with the guiding questions; do Lab 1</t>
+          <t>Discuss the Chapter 1 constructivist questions; choose one and submit a 150–200-word answer within one week
+Do Lab 1</t>
         </is>
       </c>
       <c r="I4" s="74" t="inlineStr">
         <is>
-          <t>Lead the paper discussion; guide Lab 1</t>
+          <t>Lead the discussion; guide Lab 1</t>
         </is>
       </c>
       <c r="J4" s="115" t="n"/>
@@ -4659,12 +4281,12 @@
       </c>
       <c r="H5" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 2, §2.1–2.4, pp. 37–46 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 2, §2.1–2.4, pp. 37–46 before class</t>
         </is>
       </c>
       <c r="I5" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 2; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 2</t>
         </is>
       </c>
       <c r="J5" s="115" t="n"/>
@@ -4710,12 +4332,12 @@
       </c>
       <c r="H6" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 2, §2.5–2.6, pp. 47–57 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 2, §2.5–2.6, pp. 47–57 before class</t>
         </is>
       </c>
       <c r="I6" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 2; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 2</t>
         </is>
       </c>
       <c r="J6" s="115" t="n"/>
@@ -4727,8 +4349,7 @@
       </c>
       <c r="B7" s="32" t="inlineStr">
         <is>
-          <t>2.6 The relational algebra (cont.): joins, intersection, assignment, equivalent queries; division and aggregation as extended operators
-Research Corner: Codd (1970)</t>
+          <t>2.6 The relational algebra (cont.): joins, intersection, assignment, equivalent queries; division and aggregation as extended operators</t>
         </is>
       </c>
       <c r="C7" s="32" t="inlineStr">
@@ -4749,7 +4370,7 @@
       <c r="F7" s="33" t="inlineStr">
         <is>
           <t>- Slides: Chapter 2
-- Textbook: DSC Ch. 2, §2.6, pp. 48–57; Codd (1970)</t>
+- Textbook: DSC Ch. 2, §2.6, pp. 48–57</t>
         </is>
       </c>
       <c r="G7" s="33" t="inlineStr">
@@ -4761,13 +4382,13 @@
       </c>
       <c r="H7" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 2, §2.6, pp. 48–57; Codd (1970) before class; prepare the constructivist questions
+          <t>Read DSC Ch. 2, §2.6, pp. 48–57 before class
 Self-study: Relational calculus (tuple and domain) and Codd's theorem, DSC online Ch. 27 – guided reading with worksheet</t>
         </is>
       </c>
       <c r="I7" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 2; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 2</t>
         </is>
       </c>
       <c r="J7" s="115" t="n"/>
@@ -4859,12 +4480,13 @@
       </c>
       <c r="H9" s="31" t="inlineStr">
         <is>
-          <t>Submit the self-study worksheet; solve the proof exercises</t>
+          <t>Submit the self-study worksheet; solve the proof exercises
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I9" s="74" t="inlineStr">
         <is>
-          <t>Check the worksheet; discuss common mistakes</t>
+          <t>Check the worksheet; discuss common mistakes; lead the discussion of the constructivist questions</t>
         </is>
       </c>
       <c r="J9" s="115" t="inlineStr">
@@ -4919,12 +4541,12 @@
       </c>
       <c r="H10" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 3, §3.1–3.3, pp. 65–78 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 3, §3.1–3.3, pp. 65–78 before class</t>
         </is>
       </c>
       <c r="I10" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 3; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 3</t>
         </is>
       </c>
       <c r="J10" s="115" t="n"/>
@@ -4971,12 +4593,12 @@
       </c>
       <c r="H11" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 3, §3.4–3.6, pp. 79–90 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 3, §3.4–3.6, pp. 79–90 before class</t>
         </is>
       </c>
       <c r="I11" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 3; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 3</t>
         </is>
       </c>
       <c r="J11" s="115" t="n"/>
@@ -5026,26 +4648,25 @@
       </c>
       <c r="H12" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 3, §3.7–3.8, pp. 91–107 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 3, §3.7–3.8, pp. 91–107 before class</t>
         </is>
       </c>
       <c r="I12" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 3; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 3</t>
         </is>
       </c>
       <c r="J12" s="115" t="n"/>
       <c r="K12" s="115" t="n"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="42" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="32" t="inlineStr">
         <is>
           <t>3.9 Modification of the database
-Semantics of SQL: bag semantics and translation to relational algebra
-Research Corner: Chamberlin &amp; Boyce (1974)</t>
+Semantics of SQL: bag semantics and translation to relational algebra</t>
         </is>
       </c>
       <c r="C13" s="32" t="inlineStr">
@@ -5066,7 +4687,7 @@
       <c r="F13" s="33" t="inlineStr">
         <is>
           <t>- Slides: Chapter 3
-- Textbook: DSC Ch. 3, §3.9, pp. 108–113; Chamberlin &amp; Boyce (1974)</t>
+- Textbook: DSC Ch. 3, §3.9, pp. 108–113</t>
         </is>
       </c>
       <c r="G13" s="33" t="inlineStr">
@@ -5078,7 +4699,8 @@
       </c>
       <c r="H13" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 3, §3.9, pp. 108–113; Chamberlin &amp; Boyce (1974) before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 3, §3.9, pp. 108–113 before class
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I13" s="74" t="inlineStr">
@@ -5229,12 +4851,12 @@
       </c>
       <c r="H16" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 4, §4.1–4.2, pp. 125–142 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 4, §4.1–4.2, pp. 125–142 before class</t>
         </is>
       </c>
       <c r="I16" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 4; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 4</t>
         </is>
       </c>
       <c r="J16" s="115" t="inlineStr">
@@ -5289,13 +4911,13 @@
       </c>
       <c r="H17" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 4, §4.3–4.5, pp. 143–163 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 4, §4.3–4.5, pp. 143–163 before class
 Self-study: DSC §4.7 Authorization, pp. 165–172</t>
         </is>
       </c>
       <c r="I17" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 4; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 4</t>
         </is>
       </c>
       <c r="J17" s="115" t="n"/>
@@ -5341,13 +4963,13 @@
       </c>
       <c r="H18" s="31" t="inlineStr">
         <is>
-          <t>Read DSC §4.6, p. 164; §5.4, pp. 213–218 before class; prepare the constructivist questions
+          <t>Read DSC §4.6, p. 164; §5.4, pp. 213–218 before class
 Self-study: DSC §5.5 Advanced aggregation features (ranking, windowing), pp. 219–230</t>
         </is>
       </c>
       <c r="I18" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 4; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 4</t>
         </is>
       </c>
       <c r="J18" s="115" t="n"/>
@@ -5393,8 +5015,9 @@
       </c>
       <c r="H19" s="31" t="inlineStr">
         <is>
-          <t>Read DSC §5.1, pp. 183–197 before class; prepare the constructivist questions
-Self-study: DSC §9.8 Application security, pp. 437–446; optional: §5.2–5.3 functions, procedures, triggers, pp. 198–212</t>
+          <t>Read DSC §5.1, pp. 183–197 before class
+Self-study: DSC §9.8 Application security, pp. 437–446; optional: §5.2–5.3 functions, procedures, triggers, pp. 198–212
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I19" s="74" t="inlineStr">
@@ -5543,12 +5166,12 @@
       </c>
       <c r="H22" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 6, §6.1–6.3, pp. 241–251 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 6, §6.1–6.3, pp. 241–251 before class</t>
         </is>
       </c>
       <c r="I22" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 5; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 5</t>
         </is>
       </c>
       <c r="J22" s="115" t="n"/>
@@ -5595,12 +5218,12 @@
       </c>
       <c r="H23" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 6, §6.4–6.6, pp. 252–263 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 6, §6.4–6.6, pp. 252–263 before class</t>
         </is>
       </c>
       <c r="I23" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 5; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 5</t>
         </is>
       </c>
       <c r="J23" s="115" t="n"/>
@@ -5645,13 +5268,13 @@
       </c>
       <c r="H24" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 6, §6.7, pp. 264–270 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 6, §6.7, pp. 264–270 before class
 Self-study: DSC §6.8 Extended E-R features, pp. 271–278</t>
         </is>
       </c>
       <c r="I24" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 5; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 5</t>
         </is>
       </c>
       <c r="J24" s="115" t="n"/>
@@ -5663,8 +5286,7 @@
       </c>
       <c r="B25" s="32" t="inlineStr">
         <is>
-          <t>6.9 Entity-relationship design issues; limits of the E-R model
-Research Corner: Chen (1976)</t>
+          <t>6.9 Entity-relationship design issues; limits of the E-R model</t>
         </is>
       </c>
       <c r="C25" s="32" t="inlineStr">
@@ -5685,7 +5307,7 @@
       <c r="F25" s="33" t="inlineStr">
         <is>
           <t>- Slides: Chapter 5
-- Textbook: DSC Ch. 6, §6.9, pp. 279–284; Chen (1976)</t>
+- Textbook: DSC Ch. 6, §6.9, pp. 279–284</t>
         </is>
       </c>
       <c r="G25" s="31" t="inlineStr">
@@ -5697,8 +5319,9 @@
       </c>
       <c r="H25" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 6, §6.9, pp. 279–284; Chen (1976) before class; prepare the constructivist questions
-Self-study: DSC §6.10–6.11 Alternative notations (crow's foot, UML) and other aspects of design, pp. 285–291</t>
+          <t>Read DSC Ch. 6, §6.9, pp. 279–284 before class
+Self-study: DSC §6.10–6.11 Alternative notations (crow's foot, UML) and other aspects of design, pp. 285–291
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I25" s="74" t="inlineStr">
@@ -5800,12 +5423,12 @@
       </c>
       <c r="H27" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 7, §7.1–7.2, pp. 303–312 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 7, §7.1–7.2, pp. 303–312 before class</t>
         </is>
       </c>
       <c r="I27" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 6</t>
         </is>
       </c>
       <c r="J27" s="115" t="n"/>
@@ -5850,12 +5473,12 @@
       </c>
       <c r="H28" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 7, §7.3, pp. 313–319 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 7, §7.3, pp. 313–319 before class</t>
         </is>
       </c>
       <c r="I28" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 6</t>
         </is>
       </c>
       <c r="J28" s="115" t="n"/>
@@ -5900,12 +5523,12 @@
       </c>
       <c r="H29" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class</t>
         </is>
       </c>
       <c r="I29" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 6</t>
         </is>
       </c>
       <c r="J29" s="115" t="n"/>
@@ -5950,12 +5573,12 @@
       </c>
       <c r="H30" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class</t>
         </is>
       </c>
       <c r="I30" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 6</t>
         </is>
       </c>
       <c r="J30" s="115" t="n"/>
@@ -6000,26 +5623,25 @@
       </c>
       <c r="H31" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 7, §7.5, pp. 330–335 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 7, §7.5, pp. 330–335 before class</t>
         </is>
       </c>
       <c r="I31" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 6</t>
         </is>
       </c>
       <c r="J31" s="115" t="n"/>
       <c r="K31" s="115" t="n"/>
     </row>
-    <row r="32" ht="60" customHeight="1">
+    <row r="32" ht="45" customHeight="1">
       <c r="A32" s="42" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
           <t>7.6 Decomposition using multivalued dependencies (4NF, overview)
-7.8 Atomic domains and first normal form
-Research Corner: Kent (1983)</t>
+7.8 Atomic domains and first normal form</t>
         </is>
       </c>
       <c r="C32" s="32" t="inlineStr">
@@ -6052,8 +5674,9 @@
       </c>
       <c r="H32" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 7, §7.6, §7.8, pp. 336–340, 342 before class; prepare the constructivist questions
-Self-study: DSC §7.7 More normal forms, p. 341; §7.9 Database-design process, pp. 343–346</t>
+          <t>Read DSC Ch. 7, §7.6, §7.8, pp. 336–340, 342 before class
+Self-study: DSC §7.7 More normal forms, p. 341; §7.9 Database-design process, pp. 343–346
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I32" s="74" t="inlineStr">
@@ -6250,13 +5873,13 @@
       </c>
       <c r="H36" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 13, §13.1–13.3, pp. 587–601 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 13, §13.1–13.3, pp. 587–601 before class
 Self-study: DSC §12.1 Physical storage media, pp. 559–561; §12.6 Disk-block access, pp. 577–579</t>
         </is>
       </c>
       <c r="I36" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 7; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 7</t>
         </is>
       </c>
       <c r="J36" s="115" t="n"/>
@@ -6303,13 +5926,13 @@
       </c>
       <c r="H37" s="31" t="inlineStr">
         <is>
-          <t>Read DSC §13.5, pp. 604–610; Ch. 14, §14.1–14.2, pp. 623–633 before class; prepare the constructivist questions
+          <t>Read DSC §13.5, pp. 604–610; Ch. 14, §14.1–14.2, pp. 623–633 before class
 Self-study: DSC §13.4 Data-dictionary storage, pp. 602–603</t>
         </is>
       </c>
       <c r="I37" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 7; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 7</t>
         </is>
       </c>
       <c r="J37" s="115" t="n"/>
@@ -6354,19 +5977,19 @@
       </c>
       <c r="H38" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 14, §14.3, pp. 634–649 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 14, §14.3, pp. 634–649 before class
 Self-study: DSC §14.4 B+-tree extensions, pp. 650–657</t>
         </is>
       </c>
       <c r="I38" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 7; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 7</t>
         </is>
       </c>
       <c r="J38" s="115" t="n"/>
       <c r="K38" s="115" t="n"/>
     </row>
-    <row r="39" ht="75" customHeight="1">
+    <row r="39" ht="60" customHeight="1">
       <c r="A39" s="42" t="n">
         <v>38</v>
       </c>
@@ -6374,8 +5997,7 @@
         <is>
           <t>14.5 Hash indices
 14.6 Multiple-key access
-14.7 Creation of indices
-Research Corner: Bayer &amp; McCreight (1972); Kraska et al. (2018)</t>
+14.7 Creation of indices</t>
         </is>
       </c>
       <c r="C39" s="32" t="inlineStr">
@@ -6408,13 +6030,13 @@
       </c>
       <c r="H39" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 14, §14.5–14.7, pp. 658–664 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 14, §14.5–14.7, pp. 658–664 before class
 Self-study: Optional: §13.6 Column-oriented storage, pp. 611–614; §14.8 Write-optimized index structures (LSM), pp. 665–669</t>
         </is>
       </c>
       <c r="I39" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 7; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 7</t>
         </is>
       </c>
       <c r="J39" s="115" t="n"/>
@@ -6457,12 +6079,13 @@
       </c>
       <c r="H40" s="31" t="inlineStr">
         <is>
-          <t>Solve the exercises; compare hand-computed costs with the formulas</t>
+          <t>Solve the exercises; compare hand-computed costs with the formulas
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I40" s="74" t="inlineStr">
         <is>
-          <t>Guide the exercises; discuss solutions</t>
+          <t>Guide the exercises; discuss solutions; lead the discussion of the constructivist questions</t>
         </is>
       </c>
       <c r="J40" s="115" t="n"/>
@@ -6557,12 +6180,12 @@
       </c>
       <c r="H42" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 15, §15.1–15.3, pp. 689–700 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 15, §15.1–15.3, pp. 689–700 before class</t>
         </is>
       </c>
       <c r="I42" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 8; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 8</t>
         </is>
       </c>
       <c r="J42" s="115" t="n"/>
@@ -6608,12 +6231,12 @@
       </c>
       <c r="H43" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 15, §15.4, pp. 701–703; §15.5, pp. 704–718 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 15, §15.4, pp. 701–703; §15.5, pp. 704–718 before class</t>
         </is>
       </c>
       <c r="I43" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 8; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 8</t>
         </is>
       </c>
       <c r="J43" s="115" t="n"/>
@@ -6658,13 +6281,13 @@
       </c>
       <c r="H44" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 15, §15.5, pp. 704–718 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 15, §15.5, pp. 704–718 before class
 Self-study: DSC §15.6 Other operations, pp. 719–723; §15.7 Evaluation of expressions (pipelining), pp. 724–730</t>
         </is>
       </c>
       <c r="I44" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 8; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 8</t>
         </is>
       </c>
       <c r="J44" s="115" t="n"/>
@@ -6710,12 +6333,12 @@
       </c>
       <c r="H45" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 16, §16.1–16.2, pp. 743–756 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 16, §16.1–16.2, pp. 743–756 before class</t>
         </is>
       </c>
       <c r="I45" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 8; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 8</t>
         </is>
       </c>
       <c r="J45" s="115" t="n"/>
@@ -6727,8 +6350,7 @@
       </c>
       <c r="B46" s="32" t="inlineStr">
         <is>
-          <t>16.4 Choice of evaluation plans: cost-based join ordering (dynamic programming)
-Research Corner: Selinger et al. (1979)</t>
+          <t>16.4 Choice of evaluation plans: cost-based join ordering (dynamic programming)</t>
         </is>
       </c>
       <c r="C46" s="32" t="inlineStr">
@@ -6761,8 +6383,9 @@
       </c>
       <c r="H46" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 16, §16.4, pp. 766–777 before class; prepare the constructivist questions
-Self-study: DSC §16.3 Estimating statistics of expression results, pp. 757–765</t>
+          <t>Read DSC Ch. 16, §16.4, pp. 766–777 before class
+Self-study: DSC §16.3 Estimating statistics of expression results, pp. 757–765
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I46" s="74" t="inlineStr">
@@ -6865,12 +6488,12 @@
       </c>
       <c r="H48" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 17, §17.1–17.4, pp. 799–806 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 17, §17.1–17.4, pp. 799–806 before class</t>
         </is>
       </c>
       <c r="I48" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J48" s="115" t="n"/>
@@ -6916,12 +6539,12 @@
       </c>
       <c r="H49" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 17, §17.5–17.6, pp. 807–818 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 17, §17.5–17.6, pp. 807–818 before class</t>
         </is>
       </c>
       <c r="I49" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J49" s="115" t="n"/>
@@ -6969,12 +6592,12 @@
       </c>
       <c r="H50" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 17, §17.7–17.10, pp. 819–827 before class; prepare the constructivist questions</t>
+          <t>Read DSC Ch. 17, §17.7–17.10, pp. 819–827 before class</t>
         </is>
       </c>
       <c r="I50" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J50" s="115" t="n"/>
@@ -7019,13 +6642,13 @@
       </c>
       <c r="H51" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 18, §18.1, pp. 835–848 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 18, §18.1, pp. 835–848 before class
 Self-study: DSC §18.3 Multiple granularity, pp. 853–856</t>
         </is>
       </c>
       <c r="I51" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J51" s="115" t="n"/>
@@ -7071,13 +6694,13 @@
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 18, §18.2, pp. 849–852; §18.4, pp. 857–860 before class; prepare the constructivist questions
+          <t>Read DSC Ch. 18, §18.2, pp. 849–852; §18.4, pp. 857–860 before class
 Self-study: DSC §18.5 Timestamp-based protocols, pp. 861–865; §18.7 Multiversion schemes, pp. 869–871</t>
         </is>
       </c>
       <c r="I52" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J52" s="115" t="n"/>
@@ -7089,8 +6712,7 @@
       </c>
       <c r="B53" s="32" t="inlineStr">
         <is>
-          <t>18.8 Snapshot isolation and write skew
-Research Corner: Berenson et al. (1995)</t>
+          <t>18.8 Snapshot isolation and write skew</t>
         </is>
       </c>
       <c r="C53" s="32" t="inlineStr">
@@ -7111,7 +6733,7 @@
       <c r="F53" s="31" t="inlineStr">
         <is>
           <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 18, §18.8, pp. 872–879; Berenson et al. (1995)</t>
+- Textbook: DSC Ch. 18, §18.8, pp. 872–879</t>
         </is>
       </c>
       <c r="G53" s="31" t="inlineStr">
@@ -7123,8 +6745,9 @@
       </c>
       <c r="H53" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 18, §18.8, pp. 872–879; Berenson et al. (1995) before class; prepare the constructivist questions
-Self-study: DSC §18.9 Weak levels of consistency in practice, pp. 880–882</t>
+          <t>Read DSC Ch. 18, §18.8, pp. 872–879 before class
+Self-study: DSC §18.9 Weak levels of consistency in practice, pp. 880–882
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I53" s="74" t="inlineStr">
@@ -7224,8 +6847,9 @@
       </c>
       <c r="H55" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 19, §19.1, §19.3, pp. 907, 912–921 before class; prepare the constructivist questions
-Self-study: DSC §19.2 Storage, pp. 908–911; §19.4 Recovery algorithm, pp. 922–925; §19.5–19.6, pp. 926–930; optional §19.9 ARIES, pp. 941–946</t>
+          <t>Read DSC Ch. 19, §19.1, §19.3, pp. 907, 912–921 before class
+Self-study: DSC §19.2 Storage, pp. 908–911; §19.4 Recovery algorithm, pp. 922–925; §19.5–19.6, pp. 926–930; optional §19.9 ARIES, pp. 941–946
+Discuss this chapter's constructivist questions; choose one and submit a 150–200-word answer within one week</t>
         </is>
       </c>
       <c r="I55" s="74" t="inlineStr">
@@ -7639,7 +7263,7 @@
       </c>
       <c r="B2" s="71" t="inlineStr">
         <is>
-          <t>Research labs</t>
+          <t>Labs and constructivist questions</t>
         </is>
       </c>
       <c r="C2" s="69" t="inlineStr">
@@ -7651,42 +7275,44 @@
         <v>10</v>
       </c>
       <c r="E2" s="69" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F2" s="69" t="n">
         <v>0.0001</v>
       </c>
       <c r="G2" s="19" t="inlineStr">
         <is>
-          <t>In lab sessions</t>
+          <t>Labs: in lab sessions; CQ answers: 1 week after each discussion</t>
         </is>
       </c>
       <c r="H2" s="72" t="inlineStr">
         <is>
-          <t>CLO2, CLO3, CLO4, CLO5, CLO6, CLO7, CLO8</t>
+          <t>CLO1, CLO2, CLO3, CLO4, CLO5, CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>Lab exercises, Python implementations with tests, 'Investigate' mini-reports</t>
-        </is>
-      </c>
-      <c r="J2" s="27" t="n">
-        <v>9</v>
+          <t>Lab exercises, Python implementations with tests, 'Investigate' mini-reports; short written answers to constructivist questions</t>
+        </is>
+      </c>
+      <c r="J2" s="27" t="inlineStr">
+        <is>
+          <t>9 labs + 10 CQ answers</t>
+        </is>
       </c>
       <c r="K2" s="28" t="inlineStr">
         <is>
-          <t>Labs 1–9 (Chapters 1–9)</t>
+          <t>Labs 1–9 (Chapters 1–9); one constructivist question chosen by the student from each of the 10 chapters</t>
         </is>
       </c>
       <c r="L2" s="19" t="inlineStr">
         <is>
-          <t>in class, by instructor</t>
+          <t>labs: in class, by instructor; CQ answers: on the LMS, by instructor with a short rubric</t>
         </is>
       </c>
       <c r="M2" s="25" t="inlineStr">
         <is>
-          <t>Each lab is worth about 1.1% (10% / 9). The 'Investigate' part (hypothesis, experiment, evidence) counts for at least 40% of each lab mark. Python tasks are graded by the provided unit tests and by code review.</t>
+          <t>Labs 6% in total (about 0.67% each). Constructivist-question answers 4% in total (0.4% each; 150–200 words; graded on reasoning, use of the textbook and clarity). The 'Investigate' part (hypothesis, experiment, evidence) counts for at least 40% of each lab mark. Python tasks are graded by the provided unit tests and by code review.</t>
         </is>
       </c>
       <c r="N2" s="71" t="inlineStr">
@@ -7935,8 +7561,8 @@
       </c>
       <c r="K6" s="28" t="inlineStr">
         <is>
-          <t>- cover Chapters 6–10 (DSC Ch. 7, 12–19) and the Research Corner papers
-- topics: empirical studies (indexes, join algorithms, isolation levels), algorithm implementation and evaluation (FD algorithms, serializability, relational algebra), or reproducing a result from a paper</t>
+          <t>- cover Chapters 6–10 (DSC Ch. 7, 12–19)
+- topics: empirical studies (indexes, join algorithms, isolation levels), algorithm implementation and evaluation (FD algorithms, serializability, relational algebra), or reproducing at small scale a result from a published paper found by the group</t>
         </is>
       </c>
       <c r="L6" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Use the rewritten course objectives as the syllabus Description
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0157NQpBHkydaVuWPpDtVnkB
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -1583,7 +1583,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="125" customFormat="1" customHeight="1" s="10">
+    <row r="12" ht="150" customFormat="1" customHeight="1" s="10">
       <c r="A12" s="78" t="n">
         <v>11</v>
       </c>
@@ -1596,12 +1596,12 @@
       <c r="C12" s="17" t="inlineStr">
         <is>
           <t>This course aims to help students:
-- understand the basic concepts of database systems and the relational model;
+- understand the formal foundations of the relational model: relations as sets, and keys and constraints as logical statements;
 - design databases with the Entity-Relationship model and convert them into relational schemas;
-- write queries in relational algebra, relational calculus and SQL;
-- use functional dependencies to evaluate and normalize a database design;
-- explain how a DBMS stores data, uses indexes and processes queries;
-- explain how transactions, concurrency control and recovery keep data correct;
+- write queries in relational algebra, relational calculus and SQL, and reason about what each language can express;
+- apply functional-dependency theory and its algorithms to normalize a design, and prove that a decomposition is correct;
+- analyze the cost and complexity of storage, indexing and query-processing algorithms;
+- explain the system internals that keep data correct: transactions, concurrency control and recovery;
 - answer research-style questions and carry out small experiments on database topics.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add a T-SQL programming chapter by trimming the internals chapters
New chapter C5 (sessions 20-25): T-SQL functions, stored procedures,
triggers and cursors, with Lab 3 in two parts. Storage/indexing, query
processing and transactions/recovery go from 20 to 14 sessions; join
ordering by dynamic programming becomes optional self-study and
snapshot isolation an overview. Still 60 sessions, 5 labs, 2 progress
tests and one group project. CLO4, CQs, grading scopes, the council
brief and the project notes are updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsfsusx3YZQC9pVr8xoQKL
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -1599,8 +1599,9 @@
 - Understand the formal foundations of the relational model: relations as sets, and keys and constraints as logical statements;
 - Design databases with the Entity-Relationship model and convert them into relational schemas;
 - Write queries in relational algebra, relational calculus and SQL, and reason about what each language can express;
+- Program the database server in T-SQL (functions, stored procedures, triggers and cursors), and compare row-by-row with set-based processing;
 - Apply functional-dependency theory and its algorithms to normalize a design, and prove that a decomposition is correct;
-- Analyze the cost and complexity of storage, indexing and query-processing algorithms;
+- Analyze the cost of storage, indexing and query-processing algorithms;
 - Explain the system internals that keep data correct: transactions, concurrency control and recovery;
 - Answer research-style questions and carry out small experiments on database topics.</t>
         </is>
@@ -2259,7 +2260,7 @@
       </c>
       <c r="C5" s="104" t="inlineStr">
         <is>
-          <t>Use SQL to define, populate, modify and query relational databases (joins, aggregation, subqueries, views, parameterized queries) and explain query results through SQL semantics (three-valued logic; bag semantics through guided self-study).</t>
+          <t>Use SQL to define, populate, modify and query relational databases (joins, aggregation, subqueries, views, parameterized queries), program the database server in T-SQL (user-defined functions, stored procedures, triggers, cursors), and explain query results through SQL semantics (three-valued logic; bag semantics through guided self-study).</t>
         </is>
       </c>
       <c r="D5" s="103" t="n"/>
@@ -3170,7 +3171,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="135" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C14" s="136" t="inlineStr">
         <is>
@@ -3179,7 +3180,7 @@
       </c>
       <c r="D14" s="137" t="inlineStr">
         <is>
-          <t>Why is a grade an attribute of the enrollment relationship and not of STUDENT or SECTION? What goes wrong if it is placed on either entity?</t>
+          <t>A business rule can often be enforced by a CHECK constraint, a trigger or a stored procedure. Which would you choose, and why does the declarative option usually win when it is possible?</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3189,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="135" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" s="136" t="inlineStr">
         <is>
@@ -3197,7 +3198,7 @@
       </c>
       <c r="D15" s="137" t="inlineStr">
         <is>
-          <t>Is a ternary relationship always equivalent to three binary relationships? Construct a counterexample.</t>
+          <t>A cursor processes one row at a time, while SQL is set-based. Why is the set-based version usually much faster, and when is a cursor still justified? Design an experiment that measures the difference.</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3207,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="135" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C16" s="136" t="inlineStr">
         <is>
@@ -3215,7 +3216,7 @@
       </c>
       <c r="D16" s="137" t="inlineStr">
         <is>
-          <t>Give a business rule of the university database that cannot be drawn in an E-R diagram. How should a designer record and enforce it?</t>
+          <t>A trigger can fire another trigger, or itself. What can go wrong with cascading triggers, and how could you argue that a given set of triggers always terminates?</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3225,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="135" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" s="136" t="inlineStr">
         <is>
@@ -3233,7 +3234,7 @@
       </c>
       <c r="D17" s="137" t="inlineStr">
         <is>
-          <t>Every normal form can be seen as removing one kind of redundancy. What single idea unifies them?</t>
+          <t>Why is a grade an attribute of the enrollment relationship and not of STUDENT or SECTION? What goes wrong if it is placed on either entity?</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3243,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="135" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" s="136" t="inlineStr">
         <is>
@@ -3251,7 +3252,7 @@
       </c>
       <c r="D18" s="137" t="inlineStr">
         <is>
-          <t>BCNF decomposition may lose a dependency. When would you accept 3NF instead, and what do you gain?</t>
+          <t>Is a ternary relationship always equivalent to three binary relationships? Construct a counterexample.</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3261,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="135" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C19" s="136" t="inlineStr">
         <is>
@@ -3269,7 +3270,7 @@
       </c>
       <c r="D19" s="137" t="inlineStr">
         <is>
-          <t>Testing whether an attribute is prime is NP-complete. What does this mean for automatic schema design tools?</t>
+          <t>Give a business rule of the university database that cannot be drawn in an E-R diagram. How should a designer record and enforce it?</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3279,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="135" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C20" s="136" t="inlineStr">
         <is>
@@ -3287,7 +3288,7 @@
       </c>
       <c r="D20" s="137" t="inlineStr">
         <is>
-          <t>Why is a B+-tree node the size of a disk block instead of holding a single key as in a binary search tree?</t>
+          <t>Every normal form can be seen as removing one kind of redundancy. What single idea unifies them?</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3297,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="135" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C21" s="136" t="inlineStr">
         <is>
@@ -3305,7 +3306,7 @@
       </c>
       <c r="D21" s="137" t="inlineStr">
         <is>
-          <t>When can a full table scan be cheaper than using an index? Design an experiment that shows it.</t>
+          <t>BCNF decomposition may lose a dependency. When would you accept 3NF instead, and what do you gain?</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3315,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="135" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C22" s="136" t="inlineStr">
         <is>
@@ -3323,7 +3324,7 @@
       </c>
       <c r="D22" s="137" t="inlineStr">
         <is>
-          <t>Could a machine-learning model replace an index? What would you need to measure to decide?</t>
+          <t>Testing whether an attribute is prime is NP-complete. What does this mean for automatic schema design tools?</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3333,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="135" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C23" s="136" t="inlineStr">
         <is>
@@ -3341,7 +3342,7 @@
       </c>
       <c r="D23" s="137" t="inlineStr">
         <is>
-          <t>The optimizer relies on estimates. What happens when the estimates are wrong, and where do the errors come from?</t>
+          <t>Why is a B+-tree node the size of a disk block instead of holding a single key as in a binary search tree?</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3351,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="135" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C24" s="136" t="inlineStr">
         <is>
@@ -3359,7 +3360,7 @@
       </c>
       <c r="D24" s="137" t="inlineStr">
         <is>
-          <t>The same query can often be written with a join, a subquery or a set operation. Should the choice affect performance? Why or why not?</t>
+          <t>When can a full table scan be cheaper than using an index? Design an experiment that shows it.</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3369,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="135" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" s="136" t="inlineStr">
         <is>
@@ -3377,7 +3378,7 @@
       </c>
       <c r="D25" s="137" t="inlineStr">
         <is>
-          <t>Why does the number of possible join orders grow so quickly, and how does dynamic programming keep the search manageable?</t>
+          <t>Could a machine-learning model replace an index? What would you need to measure to decide?</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3387,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="135" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C26" s="136" t="inlineStr">
         <is>
@@ -3395,7 +3396,7 @@
       </c>
       <c r="D26" s="137" t="inlineStr">
         <is>
-          <t>Why is serializability the accepted correctness criterion for concurrent transactions? What weaker criteria do real systems use, and why?</t>
+          <t>The optimizer relies on estimates. What happens when the estimates are wrong, and where do the errors come from?</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3405,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="135" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C27" s="136" t="inlineStr">
         <is>
@@ -3413,7 +3414,7 @@
       </c>
       <c r="D27" s="137" t="inlineStr">
         <is>
-          <t>Why does two-phase locking guarantee serializability? Explain the idea of the lock point.</t>
+          <t>The same query can often be written with a join, a subquery or a set operation. Should the choice affect performance? Why or why not?</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="135" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C28" s="136" t="inlineStr">
         <is>
@@ -3431,7 +3432,7 @@
       </c>
       <c r="D28" s="137" t="inlineStr">
         <is>
-          <t>Snapshot isolation prevents dirty reads, non-repeatable reads and phantoms. Why is it still not serializable?</t>
+          <t>Why does the number of possible join orders grow so quickly, and why can an optimizer not simply try them all?</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3450,7 @@
       </c>
       <c r="D29" s="137" t="inlineStr">
         <is>
-          <t>Why must a log record reach stable storage before the data page it describes (write-ahead logging)?</t>
+          <t>Why is serializability the accepted correctness criterion for concurrent transactions? What weaker criteria do real systems use, and why?</t>
         </is>
       </c>
     </row>
@@ -3467,7 +3468,7 @@
       </c>
       <c r="D30" s="137" t="inlineStr">
         <is>
-          <t>What would a DBMS lose, in performance and in safety, if it forced every modified page to disk at commit?</t>
+          <t>Why does two-phase locking guarantee serializability? Explain the idea of the lock point.</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3486,7 @@
       </c>
       <c r="D31" s="137" t="inlineStr">
         <is>
-          <t>Why is recovery hard to test in a lab, and how could you still gain evidence that a recovery algorithm is correct?</t>
+          <t>Why must a log record reach stable storage before the data page it describes (write-ahead logging)?</t>
         </is>
       </c>
     </row>
@@ -5014,7 +5015,7 @@
       <c r="H19" s="31" t="inlineStr">
         <is>
           <t>Read DSC §5.1, pp. 183–197 before class
-Self-study: DSC §9.8 Application security, pp. 437–446; Python access to SQL Server (pyodbc, pandas), optional; §5.2–5.3 functions, procedures, triggers, pp. 198–212, optional
+Self-study: DSC §9.8 Application security, pp. 437–446; Python access to SQL Server (pyodbc, pandas), optional
 Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
         </is>
       </c>
@@ -5080,8 +5081,7 @@
       </c>
       <c r="B21" s="32" t="inlineStr">
         <is>
-          <t>Progress test 1 (Chapters 1–4)
-Review exercises</t>
+          <t>5.2 Functions and procedures (1): T-SQL batches, variables and control flow (IF, WHILE); scalar and table-valued user-defined functions</t>
         </is>
       </c>
       <c r="C21" s="32" t="inlineStr">
@@ -5091,539 +5091,539 @@
       </c>
       <c r="D21" s="32" t="inlineStr">
         <is>
-          <t>CLO1, CLO2, CLO3, CLO4</t>
+          <t>CLO4</t>
         </is>
       </c>
       <c r="E21" s="32" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F21" s="33" t="inlineStr">
         <is>
-          <t>- Slides: Chapters 1–4
-- DSC Ch. 1–4</t>
+          <t>- Slides: Chapter 5
+- Textbook: DSC §5.2 (within pp. 198–212); T-SQL reference: control-of-flow language, CREATE FUNCTION</t>
         </is>
       </c>
       <c r="G21" s="31" t="inlineStr">
         <is>
-          <t>- Progress test 1</t>
+          <t>- Syllabus IDB201
+- Slides: Chapter 5
+- Textbook [DSC]</t>
         </is>
       </c>
       <c r="H21" s="31" t="inlineStr">
         <is>
-          <t>Review Chapters 1–4; take Progress test 1</t>
+          <t>Read DSC §5.2 (within pp. 198–212); T-SQL reference: control-of-flow language, CREATE FUNCTION before class</t>
         </is>
       </c>
       <c r="I21" s="74" t="inlineStr">
         <is>
-          <t>Run and grade Progress test 1; review the answers</t>
+          <t>Teach Chapter 5</t>
         </is>
       </c>
       <c r="J21" s="115" t="n"/>
       <c r="K21" s="115" t="n"/>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="42" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>5.2 Functions and procedures (2): stored procedures with input and output parameters; error handling with TRY...CATCH; transactions inside a procedure (preview of Chapter 10)</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>CLO4</t>
+        </is>
+      </c>
+      <c r="E22" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 5
+- Textbook: DSC §5.2 (within pp. 198–212); T-SQL reference: CREATE PROCEDURE, TRY...CATCH</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 5
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H22" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC §5.2 (within pp. 198–212); T-SQL reference: CREATE PROCEDURE, TRY...CATCH before class
+Self-study: Dynamic SQL with sp_executesql and its injection risk (T-SQL reference; links back to session 18)</t>
+        </is>
+      </c>
+      <c r="I22" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 5</t>
+        </is>
+      </c>
+      <c r="J22" s="115" t="n"/>
+      <c r="K22" s="115" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="42" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>5.3 Triggers: AFTER and INSTEAD OF triggers; the inserted and deleted tables; enforcing business rules that keys and CHECK constraints cannot express; when not to use triggers</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>CLO2, CLO4</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F23" s="33" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 5
+- Textbook: DSC §5.3 (within pp. 198–212); T-SQL reference: CREATE TRIGGER</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 5
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H23" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC §5.3 (within pp. 198–212); T-SQL reference: CREATE TRIGGER before class</t>
+        </is>
+      </c>
+      <c r="I23" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 5</t>
+        </is>
+      </c>
+      <c r="J23" s="115" t="n"/>
+      <c r="K23" s="115" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="42" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>Cursors: from the cursor concept of §5.1 to T-SQL cursors (DECLARE, OPEN, FETCH, CLOSE); row-by-row versus set-based processing, and why set-based SQL is usually faster</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>CLO4</t>
+        </is>
+      </c>
+      <c r="E24" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F24" s="33" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 5
+- Textbook: DSC §5.1 (cursors, revisited) and §5.2 (loops over query results); T-SQL reference: DECLARE CURSOR, FETCH</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 5
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H24" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC §5.1 (cursors, revisited) and §5.2 (loops over query results); T-SQL reference: DECLARE CURSOR, FETCH before class
+Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
+        </is>
+      </c>
+      <c r="I24" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 5; lead the discussion of the constructivist questions</t>
+        </is>
+      </c>
+      <c r="J24" s="115" t="n"/>
+      <c r="K24" s="115" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="42" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>Lab 3 (part 1): user-defined functions and stored procedures with parameters and error handling on the university database</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D25" s="32" t="inlineStr">
+        <is>
+          <t>CLO4</t>
+        </is>
+      </c>
+      <c r="E25" s="32" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr">
+        <is>
+          <t>- Lab 3 handout
+- Textbook: DSC Ch. 5 Exercises on §5.2; T-SQL reference</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="inlineStr">
+        <is>
+          <t>- Lab 3 handout and sample solution</t>
+        </is>
+      </c>
+      <c r="H25" s="31" t="inlineStr">
+        <is>
+          <t>Do Lab 3; submit before the end of the session</t>
+        </is>
+      </c>
+      <c r="I25" s="74" t="inlineStr">
+        <is>
+          <t>Guide Lab 3; review and grade submissions</t>
+        </is>
+      </c>
+      <c r="J25" s="115" t="n"/>
+      <c r="K25" s="115" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="42" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Lab 3 (part 2): triggers for business rules and audit logs; a cursor solution versus a set-based solution of the same task (Investigate)</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr">
+        <is>
+          <t>CLO2, CLO4, CLO8</t>
+        </is>
+      </c>
+      <c r="E26" s="32" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F26" s="33" t="inlineStr">
+        <is>
+          <t>- Lab 3 handout
+- Textbook: DSC Ch. 5 Exercises on §5.2–5.3</t>
+        </is>
+      </c>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>- Lab 3 handout and sample solution</t>
+        </is>
+      </c>
+      <c r="H26" s="31" t="inlineStr">
+        <is>
+          <t>Do Lab 3; submit before the end of the session</t>
+        </is>
+      </c>
+      <c r="I26" s="74" t="inlineStr">
+        <is>
+          <t>Guide Lab 3; review and grade submissions</t>
+        </is>
+      </c>
+      <c r="J26" s="115" t="n"/>
+      <c r="K26" s="115" t="n"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="42" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>Progress test 1 (Chapters 1–5)
+Review exercises</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="inlineStr">
+        <is>
+          <t>CLO1, CLO2, CLO3, CLO4</t>
+        </is>
+      </c>
+      <c r="E27" s="32" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F27" s="33" t="inlineStr">
+        <is>
+          <t>- Slides: Chapters 1–5
+- DSC Ch. 1–4, Ch. 5 §5.1–5.4</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="inlineStr">
+        <is>
+          <t>- Progress test 1</t>
+        </is>
+      </c>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>Review Chapters 1–5; take Progress test 1</t>
+        </is>
+      </c>
+      <c r="I27" s="74" t="inlineStr">
+        <is>
+          <t>Run and grade Progress test 1; review the answers</t>
+        </is>
+      </c>
+      <c r="J27" s="115" t="n"/>
+      <c r="K27" s="115" t="n"/>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="42" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
         <is>
           <t>6.1 Overview of the design process
 6.2 The Entity-Relationship model
 6.3 Complex attributes</t>
         </is>
       </c>
-      <c r="C22" s="32" t="inlineStr">
+      <c r="C28" s="32" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="D22" s="32" t="inlineStr">
+      <c r="D28" s="32" t="inlineStr">
         <is>
           <t>CLO2</t>
         </is>
       </c>
-      <c r="E22" s="32" t="inlineStr">
+      <c r="E28" s="32" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F22" s="33" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 5
+      <c r="F28" s="33" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 6
 - Textbook: DSC Ch. 6, §6.1–6.3, pp. 241–251</t>
         </is>
       </c>
-      <c r="G22" s="33" t="inlineStr">
+      <c r="G28" s="33" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 5
+- Slides: Chapter 6
 - Textbook [DSC]</t>
         </is>
       </c>
-      <c r="H22" s="31" t="inlineStr">
+      <c r="H28" s="31" t="inlineStr">
         <is>
           <t>Read DSC Ch. 6, §6.1–6.3, pp. 241–251 before class</t>
         </is>
       </c>
-      <c r="I22" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 5</t>
-        </is>
-      </c>
-      <c r="J22" s="115" t="n"/>
-      <c r="K22" s="115" t="n"/>
-    </row>
-    <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="42" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="32" t="inlineStr">
+      <c r="I28" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 6</t>
+        </is>
+      </c>
+      <c r="J28" s="115" t="n"/>
+      <c r="K28" s="115" t="n"/>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="42" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
         <is>
           <t>6.4 Mapping cardinalities
 6.5 Primary key
 6.6 Removing redundant attributes in entity sets</t>
         </is>
       </c>
-      <c r="C23" s="32" t="inlineStr">
+      <c r="C29" s="32" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="D23" s="32" t="inlineStr">
+      <c r="D29" s="32" t="inlineStr">
         <is>
           <t>CLO2</t>
         </is>
       </c>
-      <c r="E23" s="32" t="inlineStr">
+      <c r="E29" s="32" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F23" s="33" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 5
+      <c r="F29" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 6
 - Textbook: DSC Ch. 6, §6.4–6.6, pp. 252–263</t>
         </is>
       </c>
-      <c r="G23" s="31" t="inlineStr">
+      <c r="G29" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 5
+- Slides: Chapter 6
 - Textbook [DSC]</t>
         </is>
       </c>
-      <c r="H23" s="31" t="inlineStr">
+      <c r="H29" s="31" t="inlineStr">
         <is>
           <t>Read DSC Ch. 6, §6.4–6.6, pp. 252–263 before class</t>
         </is>
       </c>
-      <c r="I23" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 5</t>
-        </is>
-      </c>
-      <c r="J23" s="115" t="n"/>
-      <c r="K23" s="115" t="n"/>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="42" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="32" t="inlineStr">
+      <c r="I29" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 6</t>
+        </is>
+      </c>
+      <c r="J29" s="115" t="n"/>
+      <c r="K29" s="115" t="n"/>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="42" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
         <is>
           <t>6.7 Reducing E-R diagrams to relational schemas</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr">
+      <c r="C30" s="32" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="D24" s="32" t="inlineStr">
+      <c r="D30" s="32" t="inlineStr">
         <is>
           <t>CLO2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="inlineStr">
+      <c r="E30" s="32" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F24" s="33" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 5
+      <c r="F30" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 6
 - Textbook: DSC Ch. 6, §6.7, pp. 264–270</t>
         </is>
       </c>
-      <c r="G24" s="33" t="inlineStr">
+      <c r="G30" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 5
+- Slides: Chapter 6
 - Textbook [DSC]</t>
         </is>
       </c>
-      <c r="H24" s="31" t="inlineStr">
+      <c r="H30" s="31" t="inlineStr">
         <is>
           <t>Read DSC Ch. 6, §6.7, pp. 264–270 before class
 Self-study: DSC §6.8 Extended E-R features, pp. 271–278</t>
         </is>
       </c>
-      <c r="I24" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 5</t>
-        </is>
-      </c>
-      <c r="J24" s="115" t="n"/>
-      <c r="K24" s="115" t="n"/>
-    </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="42" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="32" t="inlineStr">
+      <c r="I30" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 6</t>
+        </is>
+      </c>
+      <c r="J30" s="115" t="n"/>
+      <c r="K30" s="115" t="n"/>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="42" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="32" t="inlineStr">
         <is>
           <t>6.9 Entity-relationship design issues; limits of the E-R model</t>
         </is>
       </c>
-      <c r="C25" s="32" t="inlineStr">
+      <c r="C31" s="32" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="D25" s="32" t="inlineStr">
+      <c r="D31" s="32" t="inlineStr">
         <is>
           <t>CLO2</t>
         </is>
       </c>
-      <c r="E25" s="32" t="inlineStr">
+      <c r="E31" s="32" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F25" s="33" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 5
+      <c r="F31" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 6
 - Textbook: DSC Ch. 6, §6.9, pp. 279–284</t>
         </is>
       </c>
-      <c r="G25" s="31" t="inlineStr">
+      <c r="G31" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 5
+- Slides: Chapter 6
 - Textbook [DSC]</t>
         </is>
       </c>
-      <c r="H25" s="31" t="inlineStr">
+      <c r="H31" s="31" t="inlineStr">
         <is>
           <t>Read DSC Ch. 6, §6.9, pp. 279–284 before class
 Self-study: DSC §6.10–6.11 Alternative notations (crow's foot, UML) and other aspects of design, pp. 285–291
 Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
         </is>
       </c>
-      <c r="I25" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 5; lead the discussion of the constructivist questions</t>
-        </is>
-      </c>
-      <c r="J25" s="115" t="n"/>
-      <c r="K25" s="115" t="n"/>
-    </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="42" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="32" t="inlineStr">
-        <is>
-          <t>Lab 3: E-R design, reduction to relational schemas and implementation in SQL Server</t>
-        </is>
-      </c>
-      <c r="C26" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D26" s="32" t="inlineStr">
-        <is>
-          <t>CLO2</t>
-        </is>
-      </c>
-      <c r="E26" s="32" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="F26" s="33" t="inlineStr">
-        <is>
-          <t>- Lab 3 handout
-- Textbook: DSC Ch. 6 Exercises, pp. 294–299</t>
-        </is>
-      </c>
-      <c r="G26" s="33" t="inlineStr">
-        <is>
-          <t>- Lab 3 handout and sample solution</t>
-        </is>
-      </c>
-      <c r="H26" s="31" t="inlineStr">
-        <is>
-          <t>Do Lab 3; submit before the end of the session</t>
-        </is>
-      </c>
-      <c r="I26" s="74" t="inlineStr">
-        <is>
-          <t>Guide Lab 3; review and grade submissions</t>
-        </is>
-      </c>
-      <c r="J26" s="115" t="n"/>
-      <c r="K26" s="115" t="n"/>
-    </row>
-    <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="42" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="32" t="inlineStr">
-        <is>
-          <t>7.1 Features of good relational designs: redundancy and anomalies
-7.2 Decomposition using functional dependencies</t>
-        </is>
-      </c>
-      <c r="C27" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D27" s="32" t="inlineStr">
-        <is>
-          <t>CLO5</t>
-        </is>
-      </c>
-      <c r="E27" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F27" s="33" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
-- Textbook: DSC Ch. 7, §7.1–7.2, pp. 303–312</t>
-        </is>
-      </c>
-      <c r="G27" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 6
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H27" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 7, §7.1–7.2, pp. 303–312 before class</t>
-        </is>
-      </c>
-      <c r="I27" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 6</t>
-        </is>
-      </c>
-      <c r="J27" s="115" t="n"/>
-      <c r="K27" s="115" t="n"/>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="A28" s="42" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="32" t="inlineStr">
-        <is>
-          <t>7.3 Normal forms: BCNF and 3NF</t>
-        </is>
-      </c>
-      <c r="C28" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D28" s="32" t="inlineStr">
-        <is>
-          <t>CLO5</t>
-        </is>
-      </c>
-      <c r="E28" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F28" s="33" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
-- Textbook: DSC Ch. 7, §7.3, pp. 313–319</t>
-        </is>
-      </c>
-      <c r="G28" s="33" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 6
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H28" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 7, §7.3, pp. 313–319 before class</t>
-        </is>
-      </c>
-      <c r="I28" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 6</t>
-        </is>
-      </c>
-      <c r="J28" s="115" t="n"/>
-      <c r="K28" s="115" t="n"/>
-    </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="42" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="32" t="inlineStr">
-        <is>
-          <t>7.4 Functional-dependency theory: closure of a set of FDs, Armstrong's axioms, attribute closure</t>
-        </is>
-      </c>
-      <c r="C29" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D29" s="32" t="inlineStr">
-        <is>
-          <t>CLO5</t>
-        </is>
-      </c>
-      <c r="E29" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F29" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
-- Textbook: DSC Ch. 7, §7.4, pp. 320–329</t>
-        </is>
-      </c>
-      <c r="G29" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 6
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H29" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class</t>
-        </is>
-      </c>
-      <c r="I29" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 6</t>
-        </is>
-      </c>
-      <c r="J29" s="115" t="n"/>
-      <c r="K29" s="115" t="n"/>
-    </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="42" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="32" t="inlineStr">
-        <is>
-          <t>7.4 Functional-dependency theory (cont.): canonical cover, lossless decomposition, dependency preservation; proofs of soundness</t>
-        </is>
-      </c>
-      <c r="C30" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D30" s="32" t="inlineStr">
-        <is>
-          <t>CLO5</t>
-        </is>
-      </c>
-      <c r="E30" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F30" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
-- Textbook: DSC Ch. 7, §7.4, pp. 320–329</t>
-        </is>
-      </c>
-      <c r="G30" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 6
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H30" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class</t>
-        </is>
-      </c>
-      <c r="I30" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 6</t>
-        </is>
-      </c>
-      <c r="J30" s="115" t="n"/>
-      <c r="K30" s="115" t="n"/>
-    </row>
-    <row r="31" ht="45" customHeight="1">
-      <c r="A31" s="42" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="32" t="inlineStr">
-        <is>
-          <t>7.5 Algorithms for decomposition: BCNF decomposition and 3NF synthesis</t>
-        </is>
-      </c>
-      <c r="C31" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D31" s="32" t="inlineStr">
-        <is>
-          <t>CLO5</t>
-        </is>
-      </c>
-      <c r="E31" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F31" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
-- Textbook: DSC Ch. 7, §7.5, pp. 330–335</t>
-        </is>
-      </c>
-      <c r="G31" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 6
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H31" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 7, §7.5, pp. 330–335 before class</t>
-        </is>
-      </c>
       <c r="I31" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 6</t>
+          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
         </is>
       </c>
       <c r="J31" s="115" t="n"/>
@@ -5635,363 +5635,359 @@
       </c>
       <c r="B32" s="32" t="inlineStr">
         <is>
+          <t>Lab 4: E-R design, reduction to relational schemas and implementation in SQL Server</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D32" s="32" t="inlineStr">
+        <is>
+          <t>CLO2</t>
+        </is>
+      </c>
+      <c r="E32" s="32" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F32" s="31" t="inlineStr">
+        <is>
+          <t>- Lab 4 handout
+- Textbook: DSC Ch. 6 Exercises, pp. 294–299</t>
+        </is>
+      </c>
+      <c r="G32" s="31" t="inlineStr">
+        <is>
+          <t>- Lab 4 handout and sample solution</t>
+        </is>
+      </c>
+      <c r="H32" s="31" t="inlineStr">
+        <is>
+          <t>Do Lab 4; submit before the end of the session</t>
+        </is>
+      </c>
+      <c r="I32" s="74" t="inlineStr">
+        <is>
+          <t>Guide Lab 4; review and grade submissions</t>
+        </is>
+      </c>
+      <c r="J32" s="115" t="n"/>
+      <c r="K32" s="115" t="n"/>
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="42" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>7.1 Features of good relational designs: redundancy and anomalies
+7.2 Decomposition using functional dependencies</t>
+        </is>
+      </c>
+      <c r="C33" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D33" s="32" t="inlineStr">
+        <is>
+          <t>CLO5</t>
+        </is>
+      </c>
+      <c r="E33" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F33" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 7
+- Textbook: DSC Ch. 7, §7.1–7.2, pp. 303–312</t>
+        </is>
+      </c>
+      <c r="G33" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 7
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H33" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC Ch. 7, §7.1–7.2, pp. 303–312 before class</t>
+        </is>
+      </c>
+      <c r="I33" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 7</t>
+        </is>
+      </c>
+      <c r="J33" s="115" t="n"/>
+      <c r="K33" s="115" t="n"/>
+    </row>
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="42" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>7.3 Normal forms: BCNF and 3NF</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D34" s="32" t="inlineStr">
+        <is>
+          <t>CLO5</t>
+        </is>
+      </c>
+      <c r="E34" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F34" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 7
+- Textbook: DSC Ch. 7, §7.3, pp. 313–319</t>
+        </is>
+      </c>
+      <c r="G34" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 7
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H34" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC Ch. 7, §7.3, pp. 313–319 before class</t>
+        </is>
+      </c>
+      <c r="I34" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 7</t>
+        </is>
+      </c>
+      <c r="J34" s="115" t="n"/>
+      <c r="K34" s="115" t="n"/>
+    </row>
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="42" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>7.4 Functional-dependency theory: closure of a set of FDs, Armstrong's axioms, attribute closure</t>
+        </is>
+      </c>
+      <c r="C35" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D35" s="32" t="inlineStr">
+        <is>
+          <t>CLO5</t>
+        </is>
+      </c>
+      <c r="E35" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F35" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 7
+- Textbook: DSC Ch. 7, §7.4, pp. 320–329</t>
+        </is>
+      </c>
+      <c r="G35" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 7
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H35" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class</t>
+        </is>
+      </c>
+      <c r="I35" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 7</t>
+        </is>
+      </c>
+      <c r="J35" s="115" t="n"/>
+      <c r="K35" s="115" t="n"/>
+    </row>
+    <row r="36" ht="45" customHeight="1">
+      <c r="A36" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>7.4 Functional-dependency theory (cont.): canonical cover, lossless decomposition, dependency preservation; proofs of soundness</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D36" s="32" t="inlineStr">
+        <is>
+          <t>CLO5</t>
+        </is>
+      </c>
+      <c r="E36" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F36" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 7
+- Textbook: DSC Ch. 7, §7.4, pp. 320–329</t>
+        </is>
+      </c>
+      <c r="G36" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 7
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H36" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC Ch. 7, §7.4, pp. 320–329 before class</t>
+        </is>
+      </c>
+      <c r="I36" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 7</t>
+        </is>
+      </c>
+      <c r="J36" s="115" t="n"/>
+      <c r="K36" s="115" t="n"/>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="42" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>7.5 Algorithms for decomposition: BCNF decomposition and 3NF synthesis</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D37" s="32" t="inlineStr">
+        <is>
+          <t>CLO5</t>
+        </is>
+      </c>
+      <c r="E37" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 7
+- Textbook: DSC Ch. 7, §7.5, pp. 330–335</t>
+        </is>
+      </c>
+      <c r="G37" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 7
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H37" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC Ch. 7, §7.5, pp. 330–335 before class</t>
+        </is>
+      </c>
+      <c r="I37" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 7</t>
+        </is>
+      </c>
+      <c r="J37" s="115" t="n"/>
+      <c r="K37" s="115" t="n"/>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="42" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
           <t>7.6 Decomposition using multivalued dependencies (4NF, overview)
 7.8 Atomic domains and first normal form</t>
         </is>
       </c>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="C38" s="32" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="D32" s="32" t="inlineStr">
+      <c r="D38" s="32" t="inlineStr">
         <is>
           <t>CLO5</t>
         </is>
       </c>
-      <c r="E32" s="32" t="inlineStr">
+      <c r="E38" s="32" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F32" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
+      <c r="F38" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 7
 - Textbook: DSC Ch. 7, §7.6, §7.8, pp. 336–340, 342</t>
         </is>
       </c>
-      <c r="G32" s="31" t="inlineStr">
+      <c r="G38" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 6
+- Slides: Chapter 7
 - Textbook [DSC]</t>
         </is>
       </c>
-      <c r="H32" s="31" t="inlineStr">
+      <c r="H38" s="31" t="inlineStr">
         <is>
           <t>Read DSC Ch. 7, §7.6, §7.8, pp. 336–340, 342 before class
 Self-study: DSC §7.7 More normal forms, p. 341; §7.9 Database-design process, pp. 343–346
 Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
         </is>
       </c>
-      <c r="I32" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 6; lead the discussion of the constructivist questions</t>
-        </is>
-      </c>
-      <c r="J32" s="115" t="n"/>
-      <c r="K32" s="115" t="n"/>
-    </row>
-    <row r="33" ht="45" customHeight="1">
-      <c r="A33" s="42" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="32" t="inlineStr">
-        <is>
-          <t>Guided exercises: FD theory on paper (attribute closure, candidate keys, canonical cover, BCNF and 3NF decomposition, lossless-join test)</t>
-        </is>
-      </c>
-      <c r="C33" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D33" s="32" t="inlineStr">
-        <is>
-          <t>CLO5</t>
-        </is>
-      </c>
-      <c r="E33" s="32" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="F33" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 6
-- Textbook: DSC Ch. 7 Exercises, pp. 353–359</t>
-        </is>
-      </c>
-      <c r="G33" s="31" t="inlineStr">
-        <is>
-          <t>- Exercise solutions</t>
-        </is>
-      </c>
-      <c r="H33" s="31" t="inlineStr">
-        <is>
-          <t>Solve the exercises; check each decomposition for lossless join and dependency preservation</t>
-        </is>
-      </c>
-      <c r="I33" s="74" t="inlineStr">
-        <is>
-          <t>Guide the exercises; discuss solutions</t>
-        </is>
-      </c>
-      <c r="J33" s="115" t="n"/>
-      <c r="K33" s="115" t="n"/>
-    </row>
-    <row r="34" ht="45" customHeight="1">
-      <c r="A34" s="42" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="32" t="inlineStr">
-        <is>
-          <t>Assignment milestone 1: design review (E-R model, normalized schema with constraints, research questions)</t>
-        </is>
-      </c>
-      <c r="C34" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D34" s="32" t="inlineStr">
-        <is>
-          <t>CLO2, CLO5, CLO8</t>
-        </is>
-      </c>
-      <c r="E34" s="32" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="F34" s="31" t="inlineStr">
-        <is>
-          <t>- Assignment brief and rubric</t>
-        </is>
-      </c>
-      <c r="G34" s="31" t="inlineStr">
-        <is>
-          <t>- Assignment rubric</t>
-        </is>
-      </c>
-      <c r="H34" s="31" t="inlineStr">
-        <is>
-          <t>Submit the design document; present it (5 minutes per team)</t>
-        </is>
-      </c>
-      <c r="I34" s="74" t="inlineStr">
-        <is>
-          <t>Assess the designs; give feedback</t>
-        </is>
-      </c>
-      <c r="J34" s="115" t="n"/>
-      <c r="K34" s="115" t="n"/>
-    </row>
-    <row r="35" ht="45" customHeight="1">
-      <c r="A35" s="42" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="32" t="inlineStr">
-        <is>
-          <t>Progress test 2 (Chapters 5–6)
-Review exercises</t>
-        </is>
-      </c>
-      <c r="C35" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D35" s="32" t="inlineStr">
-        <is>
-          <t>CLO2, CLO5</t>
-        </is>
-      </c>
-      <c r="E35" s="32" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="F35" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapters 5–6
-- DSC Ch. 6–7</t>
-        </is>
-      </c>
-      <c r="G35" s="31" t="inlineStr">
-        <is>
-          <t>- Progress test 2</t>
-        </is>
-      </c>
-      <c r="H35" s="31" t="inlineStr">
-        <is>
-          <t>Review Chapters 5–6; take Progress test 2</t>
-        </is>
-      </c>
-      <c r="I35" s="74" t="inlineStr">
-        <is>
-          <t>Run and grade Progress test 2; review the answers</t>
-        </is>
-      </c>
-      <c r="J35" s="115" t="n"/>
-      <c r="K35" s="115" t="n"/>
-    </row>
-    <row r="36" ht="60" customHeight="1">
-      <c r="A36" s="42" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="32" t="inlineStr">
-        <is>
-          <t>13.1 Database storage architecture
-13.2 File organization
-13.3 Organization of records in files</t>
-        </is>
-      </c>
-      <c r="C36" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D36" s="32" t="inlineStr">
-        <is>
-          <t>CLO6</t>
-        </is>
-      </c>
-      <c r="E36" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F36" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 7
-- Textbook: DSC Ch. 13, §13.1–13.3, pp. 587–601</t>
-        </is>
-      </c>
-      <c r="G36" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 7
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H36" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 13, §13.1–13.3, pp. 587–601 before class
-Self-study: DSC §12.1 Physical storage media, pp. 559–561; §12.6 Disk-block access, pp. 577–579</t>
-        </is>
-      </c>
-      <c r="I36" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 7</t>
-        </is>
-      </c>
-      <c r="J36" s="115" t="n"/>
-      <c r="K36" s="115" t="n"/>
-    </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="42" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="32" t="inlineStr">
-        <is>
-          <t>13.5 Database buffer
-14.1 Indexing: basic concepts
-14.2 Ordered indices</t>
-        </is>
-      </c>
-      <c r="C37" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D37" s="32" t="inlineStr">
-        <is>
-          <t>CLO6</t>
-        </is>
-      </c>
-      <c r="E37" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F37" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 7
-- Textbook: DSC §13.5, pp. 604–610; Ch. 14, §14.1–14.2, pp. 623–633</t>
-        </is>
-      </c>
-      <c r="G37" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 7
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H37" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC §13.5, pp. 604–610; Ch. 14, §14.1–14.2, pp. 623–633 before class
-Self-study: DSC §13.4 Data-dictionary storage, pp. 602–603</t>
-        </is>
-      </c>
-      <c r="I37" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 7</t>
-        </is>
-      </c>
-      <c r="J37" s="115" t="n"/>
-      <c r="K37" s="115" t="n"/>
-    </row>
-    <row r="38" ht="45" customHeight="1">
-      <c r="A38" s="42" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="32" t="inlineStr">
-        <is>
-          <t>14.3 B+-tree index files: structure, search, insertion, deletion; height analysis</t>
-        </is>
-      </c>
-      <c r="C38" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D38" s="32" t="inlineStr">
-        <is>
-          <t>CLO6</t>
-        </is>
-      </c>
-      <c r="E38" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F38" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 7
-- Textbook: DSC Ch. 14, §14.3, pp. 634–649</t>
-        </is>
-      </c>
-      <c r="G38" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 7
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H38" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 14, §14.3, pp. 634–649 before class
-Self-study: DSC §14.4 B+-tree extensions, pp. 650–657</t>
-        </is>
-      </c>
       <c r="I38" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 7</t>
+          <t>Teach Chapter 7; lead the discussion of the constructivist questions</t>
         </is>
       </c>
       <c r="J38" s="115" t="n"/>
       <c r="K38" s="115" t="n"/>
     </row>
-    <row r="39" ht="60" customHeight="1">
+    <row r="39" ht="45" customHeight="1">
       <c r="A39" s="42" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="32" t="inlineStr">
         <is>
-          <t>14.5 Hash indices
-14.6 Multiple-key access
-14.7 Creation of indices</t>
+          <t>Guided exercises: FD theory on paper (attribute closure, candidate keys, canonical cover, BCNF and 3NF decomposition, lossless-join test)</t>
         </is>
       </c>
       <c r="C39" s="32" t="inlineStr">
@@ -6001,36 +5997,33 @@
       </c>
       <c r="D39" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO5</t>
         </is>
       </c>
       <c r="E39" s="32" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F39" s="31" t="inlineStr">
         <is>
           <t>- Slides: Chapter 7
-- Textbook: DSC Ch. 14, §14.5–14.7, pp. 658–664</t>
+- Textbook: DSC Ch. 7 Exercises, pp. 353–359</t>
         </is>
       </c>
       <c r="G39" s="31" t="inlineStr">
         <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 7
-- Textbook [DSC]</t>
+          <t>- Exercise solutions</t>
         </is>
       </c>
       <c r="H39" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 14, §14.5–14.7, pp. 658–664 before class
-Self-study: Optional: §13.6 Column-oriented storage, pp. 611–614; §14.8 Write-optimized index structures (LSM), pp. 665–669</t>
+          <t>Solve the exercises; check each decomposition for lossless join and dependency preservation</t>
         </is>
       </c>
       <c r="I39" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 7</t>
+          <t>Guide the exercises; discuss solutions</t>
         </is>
       </c>
       <c r="J39" s="115" t="n"/>
@@ -6042,7 +6035,7 @@
       </c>
       <c r="B40" s="32" t="inlineStr">
         <is>
-          <t>Guided exercises: B+-tree insertion and deletion by hand; hashing; I/O cost of index lookups versus table scans</t>
+          <t>Assignment milestone 1: design review (E-R model, normalized schema with constraints, research questions)</t>
         </is>
       </c>
       <c r="C40" s="32" t="inlineStr">
@@ -6052,7 +6045,7 @@
       </c>
       <c r="D40" s="32" t="inlineStr">
         <is>
-          <t>CLO6</t>
+          <t>CLO2, CLO5, CLO8</t>
         </is>
       </c>
       <c r="E40" s="32" t="inlineStr">
@@ -6062,24 +6055,22 @@
       </c>
       <c r="F40" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapter 7
-- Textbook: DSC Ch. 14 Exercises, pp. 679–682</t>
+          <t>- Assignment brief and rubric</t>
         </is>
       </c>
       <c r="G40" s="31" t="inlineStr">
         <is>
-          <t>- Exercise solutions</t>
+          <t>- Assignment rubric</t>
         </is>
       </c>
       <c r="H40" s="31" t="inlineStr">
         <is>
-          <t>Solve the exercises; compare hand-computed costs with the formulas
-Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
+          <t>Submit the design document; present it (5 minutes per team)</t>
         </is>
       </c>
       <c r="I40" s="74" t="inlineStr">
         <is>
-          <t>Guide the exercises; discuss solutions; lead the discussion of the constructivist questions</t>
+          <t>Assess the designs; give feedback</t>
         </is>
       </c>
       <c r="J40" s="115" t="n"/>
@@ -6091,7 +6082,8 @@
       </c>
       <c r="B41" s="32" t="inlineStr">
         <is>
-          <t>Lab 4 (part 1): indexing experiments on a large table; logical reads with and without indexes (Investigate)</t>
+          <t>Progress test 2 (Chapters 6–7)
+Review exercises</t>
         </is>
       </c>
       <c r="C41" s="32" t="inlineStr">
@@ -6101,7 +6093,7 @@
       </c>
       <c r="D41" s="32" t="inlineStr">
         <is>
-          <t>CLO6, CLO8</t>
+          <t>CLO2, CLO5</t>
         </is>
       </c>
       <c r="E41" s="32" t="inlineStr">
@@ -6111,37 +6103,38 @@
       </c>
       <c r="F41" s="31" t="inlineStr">
         <is>
-          <t>- Lab 4 handout
-- Textbook: DSC Ch. 14 Exercises, pp. 679–682</t>
+          <t>- Slides: Chapters 6–7
+- DSC Ch. 6–7</t>
         </is>
       </c>
       <c r="G41" s="31" t="inlineStr">
         <is>
-          <t>- Lab 4 handout and sample solution</t>
+          <t>- Progress test 2</t>
         </is>
       </c>
       <c r="H41" s="31" t="inlineStr">
         <is>
-          <t>Do Lab 4; submit before the end of the session</t>
+          <t>Review Chapters 6–7; take Progress test 2</t>
         </is>
       </c>
       <c r="I41" s="74" t="inlineStr">
         <is>
-          <t>Guide Lab 4; review and grade submissions</t>
+          <t>Run and grade Progress test 2; review the answers</t>
         </is>
       </c>
       <c r="J41" s="115" t="n"/>
       <c r="K41" s="115" t="n"/>
     </row>
-    <row r="42" ht="60" customHeight="1">
+    <row r="42" ht="75" customHeight="1">
       <c r="A42" s="42" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="32" t="inlineStr">
         <is>
-          <t>15.1 Overview of query processing
-15.2 Measures of query cost
-15.3 Selection operation</t>
+          <t>13.1 Database storage architecture
+13.2 File organization
+13.3 Organization of records in files
+13.5 Database buffer</t>
         </is>
       </c>
       <c r="C42" s="32" t="inlineStr">
@@ -6162,7 +6155,7 @@
       <c r="F42" s="31" t="inlineStr">
         <is>
           <t>- Slides: Chapter 8
-- Textbook: DSC Ch. 15, §15.1–15.3, pp. 689–700</t>
+- Textbook: DSC Ch. 13, §13.1–13.3, pp. 587–601; §13.5, pp. 604–610</t>
         </is>
       </c>
       <c r="G42" s="31" t="inlineStr">
@@ -6174,7 +6167,8 @@
       </c>
       <c r="H42" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 15, §15.1–15.3, pp. 689–700 before class</t>
+          <t>Read DSC Ch. 13, §13.1–13.3, pp. 587–601; §13.5, pp. 604–610 before class
+Self-study: DSC §12.1 Physical storage media, pp. 559–561; §12.6 Disk-block access, pp. 577–579; §13.4 Data-dictionary storage, pp. 602–603</t>
         </is>
       </c>
       <c r="I42" s="74" t="inlineStr">
@@ -6185,14 +6179,15 @@
       <c r="J42" s="115" t="n"/>
       <c r="K42" s="115" t="n"/>
     </row>
-    <row r="43" ht="45" customHeight="1">
+    <row r="43" ht="60" customHeight="1">
       <c r="A43" s="42" t="n">
         <v>42</v>
       </c>
       <c r="B43" s="32" t="inlineStr">
         <is>
-          <t>15.4 Sorting (external merge sort)
-15.5 Join operation: nested-loop and block nested-loop joins</t>
+          <t>14.1 Indexing: basic concepts
+14.2 Ordered indices
+14.3 B+-tree index files: structure, search, height analysis</t>
         </is>
       </c>
       <c r="C43" s="32" t="inlineStr">
@@ -6213,7 +6208,7 @@
       <c r="F43" s="31" t="inlineStr">
         <is>
           <t>- Slides: Chapter 8
-- Textbook: DSC Ch. 15, §15.4, pp. 701–703; §15.5, pp. 704–718</t>
+- Textbook: DSC Ch. 14, §14.1–14.2, pp. 623–633; §14.3 (structure and queries), pp. 634–649</t>
         </is>
       </c>
       <c r="G43" s="31" t="inlineStr">
@@ -6225,7 +6220,7 @@
       </c>
       <c r="H43" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 15, §15.4, pp. 701–703; §15.5, pp. 704–718 before class</t>
+          <t>Read DSC Ch. 14, §14.1–14.2, pp. 623–633; §14.3 (structure and queries), pp. 634–649 before class</t>
         </is>
       </c>
       <c r="I43" s="74" t="inlineStr">
@@ -6236,13 +6231,15 @@
       <c r="J43" s="115" t="n"/>
       <c r="K43" s="115" t="n"/>
     </row>
-    <row r="44" ht="45" customHeight="1">
+    <row r="44" ht="60" customHeight="1">
       <c r="A44" s="42" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="32" t="inlineStr">
         <is>
-          <t>15.5 Join operation (cont.): indexed nested-loop, merge join, hash join; cost comparison</t>
+          <t>14.3 B+-tree index files (cont.): insertion; deletion (main idea)
+14.5 Hash indices
+14.7 Creation of indices</t>
         </is>
       </c>
       <c r="C44" s="32" t="inlineStr">
@@ -6263,7 +6260,7 @@
       <c r="F44" s="31" t="inlineStr">
         <is>
           <t>- Slides: Chapter 8
-- Textbook: DSC Ch. 15, §15.5, pp. 704–718</t>
+- Textbook: DSC Ch. 14, §14.3 (updates), pp. 634–649; §14.5–14.7, pp. 658–664</t>
         </is>
       </c>
       <c r="G44" s="31" t="inlineStr">
@@ -6275,8 +6272,8 @@
       </c>
       <c r="H44" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 15, §15.5, pp. 704–718 before class
-Self-study: DSC §15.6 Other operations, pp. 719–723; §15.7 Evaluation of expressions (pipelining), pp. 724–730</t>
+          <t>Read DSC Ch. 14, §14.3 (updates), pp. 634–649; §14.5–14.7, pp. 658–664 before class
+Self-study: DSC §14.4 B+-tree extensions, pp. 650–657; §14.6 Multiple-key access; optional: §13.6 Column-oriented storage, pp. 611–614; §14.8 Write-optimized index structures (LSM), pp. 665–669</t>
         </is>
       </c>
       <c r="I44" s="74" t="inlineStr">
@@ -6293,8 +6290,7 @@
       </c>
       <c r="B45" s="32" t="inlineStr">
         <is>
-          <t>16.1 Overview of query optimization
-16.2 Transformation of relational expressions: equivalence rules</t>
+          <t>Guided exercises: B+-tree insertion by hand; hashing; I/O cost of index lookups versus table scans</t>
         </is>
       </c>
       <c r="C45" s="32" t="inlineStr">
@@ -6309,42 +6305,44 @@
       </c>
       <c r="E45" s="32" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F45" s="31" t="inlineStr">
         <is>
           <t>- Slides: Chapter 8
-- Textbook: DSC Ch. 16, §16.1–16.2, pp. 743–756</t>
+- Textbook: DSC Ch. 14 Exercises, pp. 679–682</t>
         </is>
       </c>
       <c r="G45" s="31" t="inlineStr">
         <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 8
-- Textbook [DSC]</t>
+          <t>- Exercise solutions</t>
         </is>
       </c>
       <c r="H45" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 16, §16.1–16.2, pp. 743–756 before class</t>
+          <t>Solve the exercises; compare hand-computed costs with the formulas
+Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
         </is>
       </c>
       <c r="I45" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 8</t>
+          <t>Guide the exercises; discuss solutions; lead the discussion of the constructivist questions</t>
         </is>
       </c>
       <c r="J45" s="115" t="n"/>
       <c r="K45" s="115" t="n"/>
     </row>
-    <row r="46" ht="45" customHeight="1">
+    <row r="46" ht="75" customHeight="1">
       <c r="A46" s="42" t="n">
         <v>45</v>
       </c>
       <c r="B46" s="32" t="inlineStr">
         <is>
-          <t>16.4 Choice of evaluation plans: cost-based join ordering (dynamic programming)</t>
+          <t>15.1 Overview of query processing
+15.2 Measures of query cost
+15.3 Selection operation
+15.4 Sorting (external merge sort, main idea)</t>
         </is>
       </c>
       <c r="C46" s="32" t="inlineStr">
@@ -6364,27 +6362,25 @@
       </c>
       <c r="F46" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapter 8
-- Textbook: DSC Ch. 16, §16.4, pp. 766–777</t>
+          <t>- Slides: Chapter 9
+- Textbook: DSC Ch. 15, §15.1–15.4, pp. 689–703</t>
         </is>
       </c>
       <c r="G46" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 8
+- Slides: Chapter 9
 - Textbook [DSC]</t>
         </is>
       </c>
       <c r="H46" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 16, §16.4, pp. 766–777 before class
-Self-study: DSC §16.3 Estimating statistics of expression results, pp. 757–765
-Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
+          <t>Read DSC Ch. 15, §15.1–15.4, pp. 689–703 before class</t>
         </is>
       </c>
       <c r="I46" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 8; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J46" s="115" t="n"/>
@@ -6396,7 +6392,7 @@
       </c>
       <c r="B47" s="32" t="inlineStr">
         <is>
-          <t>Lab 4 (part 2): reading execution plans; comparing join algorithms and equivalent queries (Investigate)</t>
+          <t>15.5 Join operation: nested-loop, block nested-loop, indexed nested-loop, merge join and hash join; cost comparison</t>
         </is>
       </c>
       <c r="C47" s="32" t="inlineStr">
@@ -6406,190 +6402,192 @@
       </c>
       <c r="D47" s="32" t="inlineStr">
         <is>
-          <t>CLO6, CLO8</t>
+          <t>CLO6</t>
         </is>
       </c>
       <c r="E47" s="32" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>T</t>
         </is>
       </c>
       <c r="F47" s="31" t="inlineStr">
         <is>
-          <t>- Lab 4 handout
-- Textbook: DSC Ch. 15–16 Exercises, pp. 736–739, 789–793</t>
+          <t>- Slides: Chapter 9
+- Textbook: DSC Ch. 15, §15.5, pp. 704–718</t>
         </is>
       </c>
       <c r="G47" s="31" t="inlineStr">
         <is>
-          <t>- Lab 4 handout and sample solution</t>
+          <t>- Syllabus IDB201
+- Slides: Chapter 9
+- Textbook [DSC]</t>
         </is>
       </c>
       <c r="H47" s="31" t="inlineStr">
         <is>
-          <t>Do Lab 4; submit before the end of the session</t>
+          <t>Read DSC Ch. 15, §15.5, pp. 704–718 before class
+Self-study: DSC §15.6 Other operations, pp. 719–723; §15.7 Evaluation of expressions (pipelining), pp. 724–730</t>
         </is>
       </c>
       <c r="I47" s="74" t="inlineStr">
         <is>
-          <t>Guide Lab 4; review and grade submissions</t>
+          <t>Teach Chapter 9</t>
         </is>
       </c>
       <c r="J47" s="115" t="n"/>
       <c r="K47" s="115" t="n"/>
     </row>
-    <row r="48" ht="75" customHeight="1">
+    <row r="48" ht="60" customHeight="1">
       <c r="A48" s="42" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>16.1 Overview of query optimization
+16.2 Transformation of relational expressions: equivalence rules
+Reading execution plans in SQL Server</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D48" s="32" t="inlineStr">
+        <is>
+          <t>CLO6</t>
+        </is>
+      </c>
+      <c r="E48" s="32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F48" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 9
+- Textbook: DSC Ch. 16, §16.1–16.2, pp. 743–756</t>
+        </is>
+      </c>
+      <c r="G48" s="31" t="inlineStr">
+        <is>
+          <t>- Syllabus IDB201
+- Slides: Chapter 9
+- Textbook [DSC]</t>
+        </is>
+      </c>
+      <c r="H48" s="31" t="inlineStr">
+        <is>
+          <t>Read DSC Ch. 16, §16.1–16.2, pp. 743–756 before class
+Self-study: DSC §16.3 Estimating statistics of expression results, pp. 757–765; optional: §16.4 Choice of evaluation plans (cost-based join ordering by dynamic programming), pp. 766–777
+Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
+        </is>
+      </c>
+      <c r="I48" s="74" t="inlineStr">
+        <is>
+          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+        </is>
+      </c>
+      <c r="J48" s="115" t="n"/>
+      <c r="K48" s="115" t="n"/>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="42" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>Lab 5 (part 1): indexes and execution plans on a large table; logical reads with and without indexes; comparing join algorithms in plans (Investigate)</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="D49" s="32" t="inlineStr">
+        <is>
+          <t>CLO6, CLO8</t>
+        </is>
+      </c>
+      <c r="E49" s="32" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F49" s="31" t="inlineStr">
+        <is>
+          <t>- Lab 5 handout
+- Textbook: DSC Ch. 14–16 Exercises, pp. 679–682, 736–739, 789–793</t>
+        </is>
+      </c>
+      <c r="G49" s="31" t="inlineStr">
+        <is>
+          <t>- Lab 5 handout and sample solution</t>
+        </is>
+      </c>
+      <c r="H49" s="31" t="inlineStr">
+        <is>
+          <t>Do Lab 5; submit before the end of the session</t>
+        </is>
+      </c>
+      <c r="I49" s="74" t="inlineStr">
+        <is>
+          <t>Guide Lab 5; review and grade submissions</t>
+        </is>
+      </c>
+      <c r="J49" s="115" t="n"/>
+      <c r="K49" s="115" t="n"/>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="42" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="32" t="inlineStr">
         <is>
           <t>17.1 Transaction concept
 17.2 A simple transaction model
 17.3 Storage structure
-17.4 Transaction atomicity and durability</t>
-        </is>
-      </c>
-      <c r="C48" s="32" t="inlineStr">
+17.4 Transaction atomicity and durability
+17.10 Transactions as SQL statements</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="D48" s="32" t="inlineStr">
+      <c r="D50" s="32" t="inlineStr">
         <is>
           <t>CLO7</t>
         </is>
       </c>
-      <c r="E48" s="32" t="inlineStr">
+      <c r="E50" s="32" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F48" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 17, §17.1–17.4, pp. 799–806</t>
-        </is>
-      </c>
-      <c r="G48" s="31" t="inlineStr">
+      <c r="F50" s="31" t="inlineStr">
+        <is>
+          <t>- Slides: Chapter 10
+- Textbook: DSC Ch. 17, §17.1–17.4, pp. 799–806; §17.10</t>
+        </is>
+      </c>
+      <c r="G50" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 9
+- Slides: Chapter 10
 - Textbook [DSC]</t>
         </is>
       </c>
-      <c r="H48" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 17, §17.1–17.4, pp. 799–806 before class</t>
-        </is>
-      </c>
-      <c r="I48" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 9</t>
-        </is>
-      </c>
-      <c r="J48" s="115" t="n"/>
-      <c r="K48" s="115" t="n"/>
-    </row>
-    <row r="49" ht="45" customHeight="1">
-      <c r="A49" s="42" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="32" t="inlineStr">
-        <is>
-          <t>17.5 Transaction isolation
-17.6 Serializability: conflict serializability and precedence graphs</t>
-        </is>
-      </c>
-      <c r="C49" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D49" s="32" t="inlineStr">
-        <is>
-          <t>CLO7</t>
-        </is>
-      </c>
-      <c r="E49" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F49" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 17, §17.5–17.6, pp. 807–818</t>
-        </is>
-      </c>
-      <c r="G49" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 9
-- Textbook [DSC]</t>
-        </is>
-      </c>
-      <c r="H49" s="31" t="inlineStr">
-        <is>
-          <t>Read DSC Ch. 17, §17.5–17.6, pp. 807–818 before class</t>
-        </is>
-      </c>
-      <c r="I49" s="74" t="inlineStr">
-        <is>
-          <t>Teach Chapter 9</t>
-        </is>
-      </c>
-      <c r="J49" s="115" t="n"/>
-      <c r="K49" s="115" t="n"/>
-    </row>
-    <row r="50" ht="75" customHeight="1">
-      <c r="A50" s="42" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="32" t="inlineStr">
-        <is>
-          <t>17.7 Transaction isolation and atomicity: recoverable and cascadeless schedules
-17.8 Transaction isolation levels
-17.9 Implementation of isolation levels
-17.10 Transactions as SQL statements</t>
-        </is>
-      </c>
-      <c r="C50" s="32" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="D50" s="32" t="inlineStr">
-        <is>
-          <t>CLO7</t>
-        </is>
-      </c>
-      <c r="E50" s="32" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F50" s="31" t="inlineStr">
-        <is>
-          <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 17, §17.7–17.10, pp. 819–827</t>
-        </is>
-      </c>
-      <c r="G50" s="31" t="inlineStr">
-        <is>
-          <t>- Syllabus IDB201
-- Slides: Chapter 9
-- Textbook [DSC]</t>
-        </is>
-      </c>
       <c r="H50" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 17, §17.7–17.10, pp. 819–827 before class</t>
+          <t>Read DSC Ch. 17, §17.1–17.4, pp. 799–806; §17.10 before class</t>
         </is>
       </c>
       <c r="I50" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9</t>
+          <t>Teach Chapter 10</t>
         </is>
       </c>
       <c r="J50" s="115" t="n"/>
@@ -6601,7 +6599,8 @@
       </c>
       <c r="B51" s="32" t="inlineStr">
         <is>
-          <t>18.1 Lock-based protocols: two-phase locking and why it guarantees serializability</t>
+          <t>17.5 Transaction isolation
+17.6 Serializability: conflict serializability and precedence graphs</t>
         </is>
       </c>
       <c r="C51" s="32" t="inlineStr">
@@ -6621,39 +6620,40 @@
       </c>
       <c r="F51" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 18, §18.1, pp. 835–848</t>
+          <t>- Slides: Chapter 10
+- Textbook: DSC Ch. 17, §17.5–17.6, pp. 807–818</t>
         </is>
       </c>
       <c r="G51" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 9
+- Slides: Chapter 10
 - Textbook [DSC]</t>
         </is>
       </c>
       <c r="H51" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 18, §18.1, pp. 835–848 before class
-Self-study: DSC §18.3 Multiple granularity, pp. 853–856</t>
+          <t>Read DSC Ch. 17, §17.5–17.6, pp. 807–818 before class</t>
         </is>
       </c>
       <c r="I51" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9</t>
+          <t>Teach Chapter 10</t>
         </is>
       </c>
       <c r="J51" s="115" t="n"/>
       <c r="K51" s="115" t="n"/>
     </row>
-    <row r="52" ht="45" customHeight="1">
+    <row r="52" ht="75" customHeight="1">
       <c r="A52" s="42" t="n">
         <v>51</v>
       </c>
       <c r="B52" s="32" t="inlineStr">
         <is>
-          <t>18.2 Deadlock handling
-18.4 Insert operations, delete operations and predicate reads (phantoms)</t>
+          <t>17.7 Recoverable and cascadeless schedules
+17.8 Transaction isolation levels
+17.9 Implementation of isolation levels
+18.1 Lock-based protocols: two-phase locking (main idea, lock point)</t>
         </is>
       </c>
       <c r="C52" s="32" t="inlineStr">
@@ -6673,38 +6673,40 @@
       </c>
       <c r="F52" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 18, §18.2, pp. 849–852; §18.4, pp. 857–860</t>
+          <t>- Slides: Chapter 10
+- Textbook: DSC Ch. 17, §17.7–17.9, pp. 819–827; Ch. 18, §18.1, pp. 835–848</t>
         </is>
       </c>
       <c r="G52" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 9
+- Slides: Chapter 10
 - Textbook [DSC]</t>
         </is>
       </c>
       <c r="H52" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 18, §18.2, pp. 849–852; §18.4, pp. 857–860 before class
-Self-study: DSC §18.5 Timestamp-based protocols, pp. 861–865; §18.7 Multiversion schemes, pp. 869–871</t>
+          <t>Read DSC Ch. 17, §17.7–17.9, pp. 819–827; Ch. 18, §18.1, pp. 835–848 before class
+Self-study: DSC §18.3 Multiple granularity, pp. 853–856</t>
         </is>
       </c>
       <c r="I52" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9</t>
+          <t>Teach Chapter 10</t>
         </is>
       </c>
       <c r="J52" s="115" t="n"/>
       <c r="K52" s="115" t="n"/>
     </row>
-    <row r="53" ht="45" customHeight="1">
+    <row r="53" ht="60" customHeight="1">
       <c r="A53" s="42" t="n">
         <v>52</v>
       </c>
       <c r="B53" s="32" t="inlineStr">
         <is>
-          <t>18.8 Snapshot isolation and write skew</t>
+          <t>18.2 Deadlock handling
+18.4 Insert operations, delete operations and predicate reads (phantoms)
+18.8 Snapshot isolation (overview)</t>
         </is>
       </c>
       <c r="C53" s="32" t="inlineStr">
@@ -6724,27 +6726,26 @@
       </c>
       <c r="F53" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapter 9
-- Textbook: DSC Ch. 18, §18.8, pp. 872–879</t>
+          <t>- Slides: Chapter 10
+- Textbook: DSC Ch. 18, §18.2, pp. 849–852; §18.4, pp. 857–860; §18.8, pp. 872–879</t>
         </is>
       </c>
       <c r="G53" s="31" t="inlineStr">
         <is>
           <t>- Syllabus IDB201
-- Slides: Chapter 9
+- Slides: Chapter 10
 - Textbook [DSC]</t>
         </is>
       </c>
       <c r="H53" s="31" t="inlineStr">
         <is>
-          <t>Read DSC Ch. 18, §18.8, pp. 872–879 before class
-Self-study: DSC §18.9 Weak levels of consistency in practice, pp. 880–882
-Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
+          <t>Read DSC Ch. 18, §18.2, pp. 849–852; §18.4, pp. 857–860; §18.8, pp. 872–879 before class
+Self-study: DSC §18.5 Timestamp-based protocols, pp. 861–865; §18.7 Multiversion schemes, pp. 869–871; §18.9 Weak levels of consistency in practice, pp. 880–882</t>
         </is>
       </c>
       <c r="I53" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 9; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 10</t>
         </is>
       </c>
       <c r="J53" s="115" t="n"/>
@@ -6756,7 +6757,7 @@
       </c>
       <c r="B54" s="32" t="inlineStr">
         <is>
-          <t>Lab 5: concurrency experiments with two sessions (isolation levels, dirty reads, phantoms, deadlocks); serializability of the observed schedules by precedence graph</t>
+          <t>Lab 5 (part 2): concurrency experiments with two sessions (isolation levels, dirty reads, phantoms, deadlocks); serializability of the observed schedules by precedence graph</t>
         </is>
       </c>
       <c r="C54" s="32" t="inlineStr">
@@ -6766,7 +6767,7 @@
       </c>
       <c r="D54" s="32" t="inlineStr">
         <is>
-          <t>CLO7</t>
+          <t>CLO7, CLO8</t>
         </is>
       </c>
       <c r="E54" s="32" t="inlineStr">
@@ -6914,7 +6915,7 @@
       </c>
       <c r="D57" s="32" t="inlineStr">
         <is>
-          <t>CLO2, CLO5, CLO6, CLO7, CLO8</t>
+          <t>CLO2, CLO4, CLO5, CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="E57" s="32" t="inlineStr">
@@ -6961,7 +6962,7 @@
       </c>
       <c r="D58" s="32" t="inlineStr">
         <is>
-          <t>CLO2, CLO5, CLO6, CLO7, CLO8</t>
+          <t>CLO2, CLO4, CLO5, CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="E58" s="32" t="inlineStr">
@@ -6998,7 +6999,7 @@
       </c>
       <c r="B59" s="32" t="inlineStr">
         <is>
-          <t>Course review (part 1): Chapters 1–6, including the self-study readings</t>
+          <t>Course review (part 1): Chapters 1–7, including the self-study readings</t>
         </is>
       </c>
       <c r="C59" s="32" t="inlineStr">
@@ -7018,7 +7019,7 @@
       </c>
       <c r="F59" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapters 1–6
+          <t>- Slides: Chapters 1–7
 - Self-study reading list</t>
         </is>
       </c>
@@ -7029,7 +7030,7 @@
       </c>
       <c r="H59" s="31" t="inlineStr">
         <is>
-          <t>Review Chapters 1–6 and the self-study readings</t>
+          <t>Review Chapters 1–7 and the self-study readings</t>
         </is>
       </c>
       <c r="I59" s="74" t="inlineStr">
@@ -7046,7 +7047,7 @@
       </c>
       <c r="B60" s="32" t="inlineStr">
         <is>
-          <t>Course review (part 2): Chapters 7–10, including the self-study of recovery</t>
+          <t>Course review (part 2): Chapters 8–10, including the self-study of recovery</t>
         </is>
       </c>
       <c r="C60" s="32" t="inlineStr">
@@ -7066,7 +7067,7 @@
       </c>
       <c r="F60" s="31" t="inlineStr">
         <is>
-          <t>- Slides: Chapters 7–10
+          <t>- Slides: Chapters 8–10
 - Self-study reading list</t>
         </is>
       </c>
@@ -7077,7 +7078,7 @@
       </c>
       <c r="H60" s="31" t="inlineStr">
         <is>
-          <t>Review Chapters 7–10 and the self-study readings</t>
+          <t>Review Chapters 8–10 and the self-study readings</t>
         </is>
       </c>
       <c r="I60" s="74" t="inlineStr">
@@ -7293,7 +7294,7 @@
       </c>
       <c r="K2" s="28" t="inlineStr">
         <is>
-          <t>Labs 1–5 (Chapters 3–9: SQL queries; DDL, constraints and views; E-R design; indexing and query plans; concurrency); one constructivist question chosen by the student from each of the 10 chapters</t>
+          <t>Labs 1–5 (Chapters 3–10: SQL queries; DDL, constraints and views; T-SQL functions, procedures, triggers and cursors; E-R design; indexing, query plans and concurrency); one constructivist question chosen by the student from each of the 10 chapters</t>
         </is>
       </c>
       <c r="L2" s="19" t="inlineStr">
@@ -7357,8 +7358,8 @@
       </c>
       <c r="K3" s="28" t="inlineStr">
         <is>
-          <t>- cover Chapters 1–4 (DSC Ch. 1–4, §5.1, §5.4) and their self-study readings (relational calculus, bag semantics)
-- written items: one relational algebra/calculus proof or query, one SQL semantics question (NULL, three-valued logic)</t>
+          <t>- cover Chapters 1–5 (DSC Ch. 1–4, §5.1–5.4) and their self-study readings (relational calculus, bag semantics)
+- written items: one relational algebra/calculus proof or query, one SQL semantics or T-SQL reasoning question (NULL and three-valued logic, or the effect of a trigger)</t>
         </is>
       </c>
       <c r="L3" s="19" t="inlineStr">
@@ -7424,7 +7425,7 @@
       </c>
       <c r="K4" s="28" t="inlineStr">
         <is>
-          <t>- cover Chapters 5–6 (DSC Ch. 6–7) and their self-study sections
+          <t>- cover Chapters 6–7 (DSC Ch. 6–7) and their self-study sections
 - written items: one E-R design and reduction task, one FD proof or normalization task</t>
         </is>
       </c>
@@ -7476,7 +7477,7 @@
       </c>
       <c r="H5" s="72" t="inlineStr">
         <is>
-          <t>CLO2, CLO3, CLO5, CLO6, CLO7, CLO8</t>
+          <t>CLO2, CLO3, CLO4, CLO5, CLO6, CLO7, CLO8</t>
         </is>
       </c>
       <c r="I5" s="25" t="inlineStr">
@@ -7490,12 +7491,12 @@
       <c r="K5" s="28" t="inlineStr">
         <is>
           <t>- cover Chapters 2–10
-- each team designs one database for its own domain (E-R model, normalized schema with constraints, SQL queries with correctness arguments) and then answers research questions about it through experiments (indexes and query plans, join algorithms, isolation levels) or through constructivist questions linked to the design</t>
+- each team designs one database for its own domain (E-R model, normalized schema with constraints, SQL queries with correctness arguments, T-SQL procedures and triggers for its business rules) and then answers research questions about it through experiments (triggers versus constraints, cursors versus set-based SQL, indexes and query plans, isolation levels) or through constructivist questions linked to the design</t>
         </is>
       </c>
       <c r="L5" s="19" t="inlineStr">
         <is>
-          <t>take-home; introduced in session 7; milestone 1 (design review) in session 33; milestone 2 (progress meeting) in session 55; final presentations in sessions 56–57; graded by instructor with rubric</t>
+          <t>take-home; introduced in session 7; milestone 1 (design review) in session 39; milestone 2 (progress meeting) in session 55; final presentations in sessions 56–57; graded by instructor with rubric</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Remove constructivist questions from the T-SQL chapter
CQs are kept for the chapters that extend conceptual knowledge, so the
T-SQL skills chapter has none: 27 CQs in 9 discussion sessions, and 9
CQ answers share the 4%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsfsusx3YZQC9pVr8xoQKL
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -1621,7 +1621,7 @@
         <is>
           <t>- Students must attend at least 80% of contact slots in order to be accepted to the final examination.
 - Read the assigned textbook sections BEFORE each theory session.
-- For each chapter, choose ONE of its three constructivist questions and submit a short written answer on the LMS within one week of the discussion session. The answers are graded as part of the lab and constructivist-question score (4% in total).
+- For each chapter with constructivist questions (all chapters except C5, T-SQL programming), choose ONE of its three constructivist questions and submit a short written answer on the LMS within one week of the discussion session. The answers are graded as part of the lab and constructivist-question score (4% in total).
 - Complete all 5 labs, including the 'Investigate' part, and submit them on time.
 - Complete the group project (one assignment for the whole course): a database designed through the course and a small study answering research questions about it, delivered as an academic report, reproducible SQL scripts and a presentation.
 - Complete the guided self-study readings listed in the schedule (abstract topics such as relational calculus, bag semantics of SQL, statistics estimation and recovery algorithms); they are assessed in the progress tests and the final exam.
@@ -1665,7 +1665,7 @@
       <c r="C15" s="21" t="inlineStr">
         <is>
           <t>1) On-going Assessment:                 50%
-- 5 labs + 10 CQ answers:              10%
+- 5 labs + 9 CQ answers:                10%
 - Progress test 1:                          5%
 - Progress test 2:                          5%
 - 1 Assignment (group project):      30%
@@ -3171,7 +3171,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="135" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C14" s="136" t="inlineStr">
         <is>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="D14" s="137" t="inlineStr">
         <is>
-          <t>A business rule can often be enforced by a CHECK constraint, a trigger or a stored procedure. Which would you choose, and why does the declarative option usually win when it is possible?</t>
+          <t>Why is a grade an attribute of the enrollment relationship and not of STUDENT or SECTION? What goes wrong if it is placed on either entity?</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3189,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="135" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C15" s="136" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="D15" s="137" t="inlineStr">
         <is>
-          <t>A cursor processes one row at a time, while SQL is set-based. Why is the set-based version usually much faster, and when is a cursor still justified? Design an experiment that measures the difference.</t>
+          <t>Is a ternary relationship always equivalent to three binary relationships? Construct a counterexample.</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="135" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C16" s="136" t="inlineStr">
         <is>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="D16" s="137" t="inlineStr">
         <is>
-          <t>A trigger can fire another trigger, or itself. What can go wrong with cascading triggers, and how could you argue that a given set of triggers always terminates?</t>
+          <t>Give a business rule of the university database that cannot be drawn in an E-R diagram. How should a designer record and enforce it?</t>
         </is>
       </c>
     </row>
@@ -3225,7 +3225,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="135" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C17" s="136" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D17" s="137" t="inlineStr">
         <is>
-          <t>Why is a grade an attribute of the enrollment relationship and not of STUDENT or SECTION? What goes wrong if it is placed on either entity?</t>
+          <t>Every normal form can be seen as removing one kind of redundancy. What single idea unifies them?</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="135" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C18" s="136" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="D18" s="137" t="inlineStr">
         <is>
-          <t>Is a ternary relationship always equivalent to three binary relationships? Construct a counterexample.</t>
+          <t>BCNF decomposition may lose a dependency. When would you accept 3NF instead, and what do you gain?</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="135" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C19" s="136" t="inlineStr">
         <is>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="D19" s="137" t="inlineStr">
         <is>
-          <t>Give a business rule of the university database that cannot be drawn in an E-R diagram. How should a designer record and enforce it?</t>
+          <t>Testing whether an attribute is prime is NP-complete. What does this mean for automatic schema design tools?</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="135" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C20" s="136" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="D20" s="137" t="inlineStr">
         <is>
-          <t>Every normal form can be seen as removing one kind of redundancy. What single idea unifies them?</t>
+          <t>Why is a B+-tree node the size of a disk block instead of holding a single key as in a binary search tree?</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="135" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C21" s="136" t="inlineStr">
         <is>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="D21" s="137" t="inlineStr">
         <is>
-          <t>BCNF decomposition may lose a dependency. When would you accept 3NF instead, and what do you gain?</t>
+          <t>When can a full table scan be cheaper than using an index? Design an experiment that shows it.</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="135" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C22" s="136" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       </c>
       <c r="D22" s="137" t="inlineStr">
         <is>
-          <t>Testing whether an attribute is prime is NP-complete. What does this mean for automatic schema design tools?</t>
+          <t>Could a machine-learning model replace an index? What would you need to measure to decide?</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="135" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C23" s="136" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="D23" s="137" t="inlineStr">
         <is>
-          <t>Why is a B+-tree node the size of a disk block instead of holding a single key as in a binary search tree?</t>
+          <t>The optimizer relies on estimates. What happens when the estimates are wrong, and where do the errors come from?</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="135" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C24" s="136" t="inlineStr">
         <is>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="D24" s="137" t="inlineStr">
         <is>
-          <t>When can a full table scan be cheaper than using an index? Design an experiment that shows it.</t>
+          <t>The same query can often be written with a join, a subquery or a set operation. Should the choice affect performance? Why or why not?</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3369,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="135" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C25" s="136" t="inlineStr">
         <is>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="D25" s="137" t="inlineStr">
         <is>
-          <t>Could a machine-learning model replace an index? What would you need to measure to decide?</t>
+          <t>Why does the number of possible join orders grow so quickly, and why can an optimizer not simply try them all?</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="135" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C26" s="136" t="inlineStr">
         <is>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="D26" s="137" t="inlineStr">
         <is>
-          <t>The optimizer relies on estimates. What happens when the estimates are wrong, and where do the errors come from?</t>
+          <t>Why is serializability the accepted correctness criterion for concurrent transactions? What weaker criteria do real systems use, and why?</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="135" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C27" s="136" t="inlineStr">
         <is>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="D27" s="137" t="inlineStr">
         <is>
-          <t>The same query can often be written with a join, a subquery or a set operation. Should the choice affect performance? Why or why not?</t>
+          <t>Why does two-phase locking guarantee serializability? Explain the idea of the lock point.</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="135" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C28" s="136" t="inlineStr">
         <is>
@@ -3432,63 +3432,24 @@
       </c>
       <c r="D28" s="137" t="inlineStr">
         <is>
-          <t>Why does the number of possible join orders grow so quickly, and why can an optimizer not simply try them all?</t>
+          <t>Why must a log record reach stable storage before the data page it describes (write-ahead logging)?</t>
         </is>
       </c>
     </row>
     <row r="29" ht="13.8" customHeight="1">
-      <c r="A29" s="134" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="135" t="n">
-        <v>54</v>
-      </c>
-      <c r="C29" s="136" t="inlineStr">
-        <is>
-          <t>CQ1</t>
-        </is>
-      </c>
-      <c r="D29" s="137" t="inlineStr">
-        <is>
-          <t>Why is serializability the accepted correctness criterion for concurrent transactions? What weaker criteria do real systems use, and why?</t>
-        </is>
-      </c>
+      <c r="B29" s="96" t="n"/>
+      <c r="C29" s="96" t="n"/>
+      <c r="D29" s="97" t="n"/>
     </row>
     <row r="30" ht="13.8" customHeight="1">
-      <c r="A30" s="134" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="135" t="n">
-        <v>54</v>
-      </c>
-      <c r="C30" s="136" t="inlineStr">
-        <is>
-          <t>CQ2</t>
-        </is>
-      </c>
-      <c r="D30" s="137" t="inlineStr">
-        <is>
-          <t>Why does two-phase locking guarantee serializability? Explain the idea of the lock point.</t>
-        </is>
-      </c>
+      <c r="B30" s="96" t="n"/>
+      <c r="C30" s="96" t="n"/>
+      <c r="D30" s="97" t="n"/>
     </row>
     <row r="31" ht="13.8" customHeight="1">
-      <c r="A31" s="134" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="135" t="n">
-        <v>54</v>
-      </c>
-      <c r="C31" s="136" t="inlineStr">
-        <is>
-          <t>CQ3</t>
-        </is>
-      </c>
-      <c r="D31" s="137" t="inlineStr">
-        <is>
-          <t>Why must a log record reach stable storage before the data page it describes (write-ahead logging)?</t>
-        </is>
-      </c>
+      <c r="B31" s="96" t="n"/>
+      <c r="C31" s="96" t="n"/>
+      <c r="D31" s="97" t="n"/>
     </row>
     <row r="32" ht="13.8" customHeight="1">
       <c r="B32" s="96" t="n"/>
@@ -5265,13 +5226,12 @@
       </c>
       <c r="H24" s="31" t="inlineStr">
         <is>
-          <t>Read DSC §5.1 (cursors, revisited) and §5.2 (loops over query results); T-SQL reference: DECLARE CURSOR, FETCH before class
-Discuss this chapter's constructivist questions; choose one and submit an answer within one week</t>
+          <t>Read DSC §5.1 (cursors, revisited) and §5.2 (loops over query results); T-SQL reference: DECLARE CURSOR, FETCH before class</t>
         </is>
       </c>
       <c r="I24" s="74" t="inlineStr">
         <is>
-          <t>Teach Chapter 5; lead the discussion of the constructivist questions</t>
+          <t>Teach Chapter 5</t>
         </is>
       </c>
       <c r="J24" s="115" t="n"/>
@@ -7267,7 +7227,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="69" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="69" t="n">
         <v>0.0001</v>
@@ -7289,12 +7249,12 @@
       </c>
       <c r="J2" s="27" t="inlineStr">
         <is>
-          <t>5 labs + 10 CQ answers</t>
+          <t>5 labs + 9 CQ answers</t>
         </is>
       </c>
       <c r="K2" s="28" t="inlineStr">
         <is>
-          <t>Labs 1–5 (Chapters 3–10: SQL queries; DDL, constraints and views; T-SQL functions, procedures, triggers and cursors; E-R design; indexing, query plans and concurrency); one constructivist question chosen by the student from each of the 10 chapters</t>
+          <t>Labs 1–5 (Chapters 3–10: SQL queries; DDL, constraints and views; T-SQL functions, procedures, triggers and cursors; E-R design; indexing, query plans and concurrency); one constructivist question chosen by the student from each of the 9 chapters that have them (all except C5, T-SQL programming)</t>
         </is>
       </c>
       <c r="L2" s="19" t="inlineStr">
@@ -7304,7 +7264,7 @@
       </c>
       <c r="M2" s="25" t="inlineStr">
         <is>
-          <t>Labs 6% in total (1.2% each). Constructivist-question answers 4% in total (0.4% each; graded on reasoning, use of the textbook and clarity). The 'Investigate' part (hypothesis, experiment, evidence) counts for at least 40% of each lab mark.</t>
+          <t>Labs 6% in total (1.2% each). Constructivist-question answers 4% in total (shared equally among the 9 answers; graded on reasoning, use of the textbook and clarity). The 'Investigate' part (hypothesis, experiment, evidence) counts for at least 40% of each lab mark.</t>
         </is>
       </c>
       <c r="N2" s="71" t="inlineStr">

</xml_diff>

<commit_message>
Remove the CLO5 to PLO8 link from the syllabus
PLO8 covers programming proficiency and tools, while CLO5 is now
practised on paper only, with no lab or implementation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gQzJ9LZp5TkWfU4N1rQzM
</commit_message>
<xml_diff>
--- a/syllabus/IDB201_Syllabus.xlsx
+++ b/syllabus/IDB201_Syllabus.xlsx
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="488">
   <si>
     <t xml:space="preserve">No</t>
   </si>
@@ -3833,9 +3833,7 @@
       </c>
       <c r="G18" s="45"/>
       <c r="H18" s="45"/>
-      <c r="I18" s="58" t="s">
-        <v>112</v>
-      </c>
+      <c r="I18" s="58"/>
       <c r="J18" s="45"/>
       <c r="K18" s="57"/>
       <c r="L18" s="45"/>

</xml_diff>